<commit_message>
conf scheduling: prohibited and undesired timeslot and room tags
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="140">
   <si>
     <t>Conference name</t>
   </si>
@@ -59,18 +59,36 @@
     <t>Soft penalty per missing preferred tag in a talk's timeslot</t>
   </si>
   <si>
+    <t>Speaker undesired timeslot tag</t>
+  </si>
+  <si>
+    <t>Soft penalty per undesired tag in a talk's timeslot</t>
+  </si>
+  <si>
     <t>Talk preferred timeslot tag</t>
   </si>
   <si>
+    <t>Talk undesired timeslot tag</t>
+  </si>
+  <si>
     <t>Speaker preferred room tag</t>
   </si>
   <si>
     <t>Soft penalty per missing preferred tag in a talk's room</t>
   </si>
   <si>
+    <t>Speaker undesired room tag</t>
+  </si>
+  <si>
+    <t>Soft penalty per undesired tag in a talk's room</t>
+  </si>
+  <si>
     <t>Talk preferred room tag</t>
   </si>
   <si>
+    <t>Talk undesired room tag</t>
+  </si>
+  <si>
     <t>Day</t>
   </si>
   <si>
@@ -182,10 +200,22 @@
     <t>Preferred timeslot tags</t>
   </si>
   <si>
+    <t>Prohibited timeslot tags</t>
+  </si>
+  <si>
+    <t>Undesired timeslot tags</t>
+  </si>
+  <si>
     <t>Required room tags</t>
   </si>
   <si>
     <t>Preferred room tags</t>
+  </si>
+  <si>
+    <t>Prohibited room tags</t>
+  </si>
+  <si>
+    <t>Undesired room tags</t>
   </si>
   <si>
     <t>Amy Cole</t>
@@ -476,9 +506,9 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="29.0859375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="11.80859375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="70.88671875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="33.8671875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="12.33203125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="81.296875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -553,18 +583,18 @@
         <v>10.0</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B9" t="n">
         <v>10.0</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -575,7 +605,51 @@
         <v>10.0</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -588,130 +662,130 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="15.99609375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="6.0859375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="6.0859375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="9.41796875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="5.1484375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="16.14453125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="6.3984375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="6.32421875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="10.78515625" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="6.078125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s">
         <v>31</v>
       </c>
-      <c r="D5" t="s">
-        <v>25</v>
-      </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" t="s">
         <v>34</v>
       </c>
-      <c r="C7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" t="s">
-        <v>28</v>
-      </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -724,196 +798,196 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="6.48828125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="25.6328125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="7.109375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="26.3125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="13.6171875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -929,512 +1003,684 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="21.69921875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="22.09765625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="19.07421875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="19.47265625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="10" max="10" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="11.9453125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="24.85546875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="25.390625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="26.30859375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="26.0234375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="21.671875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="22.20703125" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="23.125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="22.84375" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="14" max="14" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" width="13.6171875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>39</v>
+        <v>64</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K3" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="L3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M3" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3" t="s">
+        <v>32</v>
+      </c>
+      <c r="O3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K4" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="L4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M4" t="s">
+        <v>32</v>
+      </c>
+      <c r="N4" t="s">
+        <v>32</v>
+      </c>
+      <c r="O4" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="F5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G5" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="H5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K5" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="L5" t="s">
+        <v>32</v>
+      </c>
+      <c r="M5" t="s">
+        <v>32</v>
+      </c>
+      <c r="N5" t="s">
+        <v>32</v>
+      </c>
+      <c r="O5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K6" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="L6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M6" t="s">
+        <v>32</v>
+      </c>
+      <c r="N6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O6" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J7" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K7" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="L7" t="s">
+        <v>32</v>
+      </c>
+      <c r="M7" t="s">
+        <v>32</v>
+      </c>
+      <c r="N7" t="s">
+        <v>32</v>
+      </c>
+      <c r="O7" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K8" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="L8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M8" t="s">
+        <v>32</v>
+      </c>
+      <c r="N8" t="s">
+        <v>32</v>
+      </c>
+      <c r="O8" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E9" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="F9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G9" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="H9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K9" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="L9" t="s">
+        <v>32</v>
+      </c>
+      <c r="M9" t="s">
+        <v>32</v>
+      </c>
+      <c r="N9" t="s">
+        <v>32</v>
+      </c>
+      <c r="O9" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G10" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="H10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K10" t="s">
-        <v>26</v>
+        <v>51</v>
+      </c>
+      <c r="L10" t="s">
+        <v>32</v>
+      </c>
+      <c r="M10" t="s">
+        <v>32</v>
+      </c>
+      <c r="N10" t="s">
+        <v>32</v>
+      </c>
+      <c r="O10" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>32</v>
+      </c>
+      <c r="H11" t="s">
+        <v>32</v>
       </c>
       <c r="I11" t="s">
-        <v>26</v>
-      </c>
-      <c r="J11" t="s">
-        <v>26</v>
-      </c>
-      <c r="K11" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M11" t="s">
+        <v>32</v>
+      </c>
+      <c r="N11" t="s">
+        <v>32</v>
+      </c>
+      <c r="O11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E12" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="F12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G12" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="H12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K12" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="L12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O12" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K13" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="L13" t="s">
+        <v>32</v>
+      </c>
+      <c r="M13" t="s">
+        <v>32</v>
+      </c>
+      <c r="N13" t="s">
+        <v>32</v>
+      </c>
+      <c r="O13" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K14" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="L14" t="s">
+        <v>32</v>
+      </c>
+      <c r="M14" t="s">
+        <v>32</v>
+      </c>
+      <c r="N14" t="s">
+        <v>32</v>
+      </c>
+      <c r="O14" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
   <mergeCells>
-    <mergeCell ref="F1:K1"/>
+    <mergeCell ref="J1:O1"/>
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -1445,972 +1691,1204 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="5.69140625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="32.125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="9.41796875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="19.3515625" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="14.375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="9.7109375" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="18.9453125" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="21.69921875" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="22.09765625" customWidth="true" bestFit="true"/>
-    <col min="10" max="10" width="19.07421875" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="19.47265625" customWidth="true" bestFit="true"/>
-    <col min="12" max="12" width="14.578125" customWidth="true" bestFit="true"/>
-    <col min="13" max="13" width="15.99609375" customWidth="true" bestFit="true"/>
-    <col min="14" max="14" width="6.0859375" customWidth="true" bestFit="true"/>
-    <col min="15" max="15" width="6.0859375" customWidth="true" bestFit="true"/>
-    <col min="16" max="16" width="6.44921875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="6.34765625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="33.1015625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.78515625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="19.83203125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="14.55078125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="11.3046875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="19.76171875" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="24.85546875" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="25.390625" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="26.30859375" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="26.0234375" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" width="21.671875" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" width="22.20703125" customWidth="true" bestFit="true"/>
+    <col min="14" max="14" width="23.125" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" width="22.84375" customWidth="true" bestFit="true"/>
+    <col min="16" max="16" width="16.65234375" customWidth="true" bestFit="true"/>
+    <col min="17" max="17" width="16.14453125" customWidth="true" bestFit="true"/>
+    <col min="18" max="18" width="6.3984375" customWidth="true" bestFit="true"/>
+    <col min="19" max="19" width="6.32421875" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="7.02734375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>18</v>
+        <v>64</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F2" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G2" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J2" t="s">
-        <v>82</v>
+        <v>32</v>
       </c>
       <c r="K2" t="s">
-        <v>26</v>
-      </c>
-      <c r="L2" t="b">
+        <v>32</v>
+      </c>
+      <c r="L2" t="s">
+        <v>92</v>
+      </c>
+      <c r="M2" t="s">
+        <v>32</v>
+      </c>
+      <c r="N2" t="s">
+        <v>32</v>
+      </c>
+      <c r="O2" t="s">
+        <v>32</v>
+      </c>
+      <c r="P2" t="b">
         <v>0</v>
       </c>
-      <c r="M2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O2" t="s">
-        <v>26</v>
-      </c>
-      <c r="P2" t="s">
-        <v>26</v>
+      <c r="Q2" t="s">
+        <v>32</v>
+      </c>
+      <c r="R2" t="s">
+        <v>32</v>
+      </c>
+      <c r="S2" t="s">
+        <v>32</v>
+      </c>
+      <c r="T2" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="B3" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F3" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G3" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="H3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J3" t="s">
-        <v>82</v>
+        <v>32</v>
       </c>
       <c r="K3" t="s">
-        <v>26</v>
-      </c>
-      <c r="L3" t="b">
+        <v>32</v>
+      </c>
+      <c r="L3" t="s">
+        <v>92</v>
+      </c>
+      <c r="M3" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3" t="s">
+        <v>32</v>
+      </c>
+      <c r="O3" t="s">
+        <v>32</v>
+      </c>
+      <c r="P3" t="b">
         <v>0</v>
       </c>
-      <c r="M3" t="s">
-        <v>26</v>
-      </c>
-      <c r="N3" t="s">
-        <v>26</v>
-      </c>
-      <c r="O3" t="s">
-        <v>26</v>
-      </c>
-      <c r="P3" t="s">
-        <v>26</v>
+      <c r="Q3" t="s">
+        <v>32</v>
+      </c>
+      <c r="R3" t="s">
+        <v>32</v>
+      </c>
+      <c r="S3" t="s">
+        <v>32</v>
+      </c>
+      <c r="T3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="E4" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="F4" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G4" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K4" t="s">
-        <v>26</v>
-      </c>
-      <c r="L4" t="b">
+        <v>32</v>
+      </c>
+      <c r="L4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M4" t="s">
+        <v>32</v>
+      </c>
+      <c r="N4" t="s">
+        <v>32</v>
+      </c>
+      <c r="O4" t="s">
+        <v>32</v>
+      </c>
+      <c r="P4" t="b">
         <v>0</v>
       </c>
-      <c r="M4" t="s">
-        <v>26</v>
-      </c>
-      <c r="N4" t="s">
-        <v>26</v>
-      </c>
-      <c r="O4" t="s">
-        <v>26</v>
-      </c>
-      <c r="P4" t="s">
-        <v>26</v>
+      <c r="Q4" t="s">
+        <v>32</v>
+      </c>
+      <c r="R4" t="s">
+        <v>32</v>
+      </c>
+      <c r="S4" t="s">
+        <v>32</v>
+      </c>
+      <c r="T4" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="E5" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="F5" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G5" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="H5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K5" t="s">
-        <v>26</v>
-      </c>
-      <c r="L5" t="b">
+        <v>32</v>
+      </c>
+      <c r="L5" t="s">
+        <v>32</v>
+      </c>
+      <c r="M5" t="s">
+        <v>32</v>
+      </c>
+      <c r="N5" t="s">
+        <v>32</v>
+      </c>
+      <c r="O5" t="s">
+        <v>32</v>
+      </c>
+      <c r="P5" t="b">
         <v>0</v>
       </c>
-      <c r="M5" t="s">
-        <v>26</v>
-      </c>
-      <c r="N5" t="s">
-        <v>26</v>
-      </c>
-      <c r="O5" t="s">
-        <v>26</v>
-      </c>
-      <c r="P5" t="s">
-        <v>26</v>
+      <c r="Q5" t="s">
+        <v>32</v>
+      </c>
+      <c r="R5" t="s">
+        <v>32</v>
+      </c>
+      <c r="S5" t="s">
+        <v>32</v>
+      </c>
+      <c r="T5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="B6" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G6" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="H6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K6" t="s">
-        <v>26</v>
-      </c>
-      <c r="L6" t="b">
+        <v>32</v>
+      </c>
+      <c r="L6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M6" t="s">
+        <v>32</v>
+      </c>
+      <c r="N6" t="s">
+        <v>32</v>
+      </c>
+      <c r="O6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P6" t="b">
         <v>0</v>
       </c>
-      <c r="M6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N6" t="s">
-        <v>26</v>
-      </c>
-      <c r="O6" t="s">
-        <v>26</v>
-      </c>
-      <c r="P6" t="s">
-        <v>26</v>
+      <c r="Q6" t="s">
+        <v>32</v>
+      </c>
+      <c r="R6" t="s">
+        <v>32</v>
+      </c>
+      <c r="S6" t="s">
+        <v>32</v>
+      </c>
+      <c r="T6" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="C7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" t="s">
+        <v>90</v>
+      </c>
+      <c r="G7" t="s">
+        <v>108</v>
+      </c>
+      <c r="H7" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" t="s">
+        <v>32</v>
+      </c>
+      <c r="J7" t="s">
+        <v>32</v>
+      </c>
+      <c r="K7" t="s">
+        <v>32</v>
+      </c>
+      <c r="L7" t="s">
+        <v>32</v>
+      </c>
+      <c r="M7" t="s">
+        <v>32</v>
+      </c>
+      <c r="N7" t="s">
+        <v>32</v>
+      </c>
+      <c r="O7" t="s">
+        <v>32</v>
+      </c>
+      <c r="P7" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q7" t="s">
         <v>28</v>
       </c>
-      <c r="D7" t="s">
-        <v>79</v>
-      </c>
-      <c r="E7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" t="s">
-        <v>80</v>
-      </c>
-      <c r="G7" t="s">
-        <v>98</v>
-      </c>
-      <c r="H7" t="s">
-        <v>26</v>
-      </c>
-      <c r="I7" t="s">
-        <v>26</v>
-      </c>
-      <c r="J7" t="s">
-        <v>26</v>
-      </c>
-      <c r="K7" t="s">
-        <v>26</v>
-      </c>
-      <c r="L7" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="M7" t="s">
-        <v>22</v>
-      </c>
-      <c r="N7" t="s">
-        <v>23</v>
-      </c>
-      <c r="O7" t="s">
-        <v>27</v>
-      </c>
-      <c r="P7" t="s">
-        <v>43</v>
+      <c r="R7" t="s">
+        <v>29</v>
+      </c>
+      <c r="S7" t="s">
+        <v>33</v>
+      </c>
+      <c r="T7" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="B8" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="E8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G8" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="H8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K8" t="s">
-        <v>26</v>
-      </c>
-      <c r="L8" t="b">
+        <v>32</v>
+      </c>
+      <c r="L8" t="s">
+        <v>32</v>
+      </c>
+      <c r="M8" t="s">
+        <v>32</v>
+      </c>
+      <c r="N8" t="s">
+        <v>32</v>
+      </c>
+      <c r="O8" t="s">
+        <v>32</v>
+      </c>
+      <c r="P8" t="b">
         <v>0</v>
       </c>
-      <c r="M8" t="s">
-        <v>26</v>
-      </c>
-      <c r="N8" t="s">
-        <v>26</v>
-      </c>
-      <c r="O8" t="s">
-        <v>26</v>
-      </c>
-      <c r="P8" t="s">
-        <v>26</v>
+      <c r="Q8" t="s">
+        <v>32</v>
+      </c>
+      <c r="R8" t="s">
+        <v>32</v>
+      </c>
+      <c r="S8" t="s">
+        <v>32</v>
+      </c>
+      <c r="T8" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="E9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G9" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="H9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J9" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K9" t="s">
-        <v>26</v>
-      </c>
-      <c r="L9" t="b">
+        <v>32</v>
+      </c>
+      <c r="L9" t="s">
+        <v>32</v>
+      </c>
+      <c r="M9" t="s">
+        <v>32</v>
+      </c>
+      <c r="N9" t="s">
+        <v>32</v>
+      </c>
+      <c r="O9" t="s">
+        <v>32</v>
+      </c>
+      <c r="P9" t="b">
         <v>0</v>
       </c>
-      <c r="M9" t="s">
-        <v>26</v>
-      </c>
-      <c r="N9" t="s">
-        <v>26</v>
-      </c>
-      <c r="O9" t="s">
-        <v>26</v>
-      </c>
-      <c r="P9" t="s">
-        <v>26</v>
+      <c r="Q9" t="s">
+        <v>32</v>
+      </c>
+      <c r="R9" t="s">
+        <v>32</v>
+      </c>
+      <c r="S9" t="s">
+        <v>32</v>
+      </c>
+      <c r="T9" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="B10" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="E10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F10" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G10" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K10" t="s">
-        <v>26</v>
-      </c>
-      <c r="L10" t="b">
+        <v>32</v>
+      </c>
+      <c r="L10" t="s">
+        <v>32</v>
+      </c>
+      <c r="M10" t="s">
+        <v>32</v>
+      </c>
+      <c r="N10" t="s">
+        <v>32</v>
+      </c>
+      <c r="O10" t="s">
+        <v>32</v>
+      </c>
+      <c r="P10" t="b">
         <v>0</v>
       </c>
-      <c r="M10" t="s">
-        <v>26</v>
-      </c>
-      <c r="N10" t="s">
-        <v>26</v>
-      </c>
-      <c r="O10" t="s">
-        <v>26</v>
-      </c>
-      <c r="P10" t="s">
-        <v>26</v>
+      <c r="Q10" t="s">
+        <v>32</v>
+      </c>
+      <c r="R10" t="s">
+        <v>32</v>
+      </c>
+      <c r="S10" t="s">
+        <v>32</v>
+      </c>
+      <c r="T10" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="B11" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F11" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G11" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="H11" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I11" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J11" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K11" t="s">
-        <v>26</v>
-      </c>
-      <c r="L11" t="b">
+        <v>32</v>
+      </c>
+      <c r="L11" t="s">
+        <v>32</v>
+      </c>
+      <c r="M11" t="s">
+        <v>32</v>
+      </c>
+      <c r="N11" t="s">
+        <v>32</v>
+      </c>
+      <c r="O11" t="s">
+        <v>32</v>
+      </c>
+      <c r="P11" t="b">
         <v>0</v>
       </c>
-      <c r="M11" t="s">
-        <v>26</v>
-      </c>
-      <c r="N11" t="s">
-        <v>26</v>
-      </c>
-      <c r="O11" t="s">
-        <v>26</v>
-      </c>
-      <c r="P11" t="s">
-        <v>26</v>
+      <c r="Q11" t="s">
+        <v>32</v>
+      </c>
+      <c r="R11" t="s">
+        <v>32</v>
+      </c>
+      <c r="S11" t="s">
+        <v>32</v>
+      </c>
+      <c r="T11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="B12" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="E12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F12" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G12" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="H12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K12" t="s">
-        <v>26</v>
-      </c>
-      <c r="L12" t="b">
+        <v>32</v>
+      </c>
+      <c r="L12" t="s">
+        <v>32</v>
+      </c>
+      <c r="M12" t="s">
+        <v>32</v>
+      </c>
+      <c r="N12" t="s">
+        <v>32</v>
+      </c>
+      <c r="O12" t="s">
+        <v>32</v>
+      </c>
+      <c r="P12" t="b">
         <v>0</v>
       </c>
-      <c r="M12" t="s">
-        <v>26</v>
-      </c>
-      <c r="N12" t="s">
-        <v>26</v>
-      </c>
-      <c r="O12" t="s">
-        <v>26</v>
-      </c>
-      <c r="P12" t="s">
-        <v>26</v>
+      <c r="Q12" t="s">
+        <v>32</v>
+      </c>
+      <c r="R12" t="s">
+        <v>32</v>
+      </c>
+      <c r="S12" t="s">
+        <v>32</v>
+      </c>
+      <c r="T12" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="B13" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="E13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F13" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G13" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K13" t="s">
-        <v>26</v>
-      </c>
-      <c r="L13" t="b">
+        <v>32</v>
+      </c>
+      <c r="L13" t="s">
+        <v>32</v>
+      </c>
+      <c r="M13" t="s">
+        <v>32</v>
+      </c>
+      <c r="N13" t="s">
+        <v>32</v>
+      </c>
+      <c r="O13" t="s">
+        <v>32</v>
+      </c>
+      <c r="P13" t="b">
         <v>0</v>
       </c>
-      <c r="M13" t="s">
-        <v>26</v>
-      </c>
-      <c r="N13" t="s">
-        <v>26</v>
-      </c>
-      <c r="O13" t="s">
-        <v>26</v>
-      </c>
-      <c r="P13" t="s">
-        <v>26</v>
+      <c r="Q13" t="s">
+        <v>32</v>
+      </c>
+      <c r="R13" t="s">
+        <v>32</v>
+      </c>
+      <c r="S13" t="s">
+        <v>32</v>
+      </c>
+      <c r="T13" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="B14" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="E14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F14" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G14" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="H14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J14" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K14" t="s">
-        <v>26</v>
-      </c>
-      <c r="L14" t="b">
+        <v>32</v>
+      </c>
+      <c r="L14" t="s">
+        <v>32</v>
+      </c>
+      <c r="M14" t="s">
+        <v>32</v>
+      </c>
+      <c r="N14" t="s">
+        <v>32</v>
+      </c>
+      <c r="O14" t="s">
+        <v>32</v>
+      </c>
+      <c r="P14" t="b">
         <v>0</v>
       </c>
-      <c r="M14" t="s">
-        <v>26</v>
-      </c>
-      <c r="N14" t="s">
-        <v>26</v>
-      </c>
-      <c r="O14" t="s">
-        <v>26</v>
-      </c>
-      <c r="P14" t="s">
-        <v>26</v>
+      <c r="Q14" t="s">
+        <v>32</v>
+      </c>
+      <c r="R14" t="s">
+        <v>32</v>
+      </c>
+      <c r="S14" t="s">
+        <v>32</v>
+      </c>
+      <c r="T14" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="B15" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D15" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="E15" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F15" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G15" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="H15" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I15" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J15" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K15" t="s">
-        <v>26</v>
-      </c>
-      <c r="L15" t="b">
+        <v>32</v>
+      </c>
+      <c r="L15" t="s">
+        <v>32</v>
+      </c>
+      <c r="M15" t="s">
+        <v>32</v>
+      </c>
+      <c r="N15" t="s">
+        <v>32</v>
+      </c>
+      <c r="O15" t="s">
+        <v>32</v>
+      </c>
+      <c r="P15" t="b">
         <v>0</v>
       </c>
-      <c r="M15" t="s">
-        <v>26</v>
-      </c>
-      <c r="N15" t="s">
-        <v>26</v>
-      </c>
-      <c r="O15" t="s">
-        <v>26</v>
-      </c>
-      <c r="P15" t="s">
-        <v>26</v>
+      <c r="Q15" t="s">
+        <v>32</v>
+      </c>
+      <c r="R15" t="s">
+        <v>32</v>
+      </c>
+      <c r="S15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T15" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="B16" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="C16" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D16" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="E16" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F16" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G16" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="H16" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I16" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J16" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K16" t="s">
-        <v>26</v>
-      </c>
-      <c r="L16" t="b">
+        <v>32</v>
+      </c>
+      <c r="L16" t="s">
+        <v>32</v>
+      </c>
+      <c r="M16" t="s">
+        <v>32</v>
+      </c>
+      <c r="N16" t="s">
+        <v>32</v>
+      </c>
+      <c r="O16" t="s">
+        <v>32</v>
+      </c>
+      <c r="P16" t="b">
         <v>0</v>
       </c>
-      <c r="M16" t="s">
-        <v>26</v>
-      </c>
-      <c r="N16" t="s">
-        <v>26</v>
-      </c>
-      <c r="O16" t="s">
-        <v>26</v>
-      </c>
-      <c r="P16" t="s">
-        <v>26</v>
+      <c r="Q16" t="s">
+        <v>32</v>
+      </c>
+      <c r="R16" t="s">
+        <v>32</v>
+      </c>
+      <c r="S16" t="s">
+        <v>32</v>
+      </c>
+      <c r="T16" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="B17" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="C17" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D17" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="E17" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F17" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G17" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="H17" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I17" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J17" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K17" t="s">
-        <v>26</v>
-      </c>
-      <c r="L17" t="b">
+        <v>32</v>
+      </c>
+      <c r="L17" t="s">
+        <v>32</v>
+      </c>
+      <c r="M17" t="s">
+        <v>32</v>
+      </c>
+      <c r="N17" t="s">
+        <v>32</v>
+      </c>
+      <c r="O17" t="s">
+        <v>32</v>
+      </c>
+      <c r="P17" t="b">
         <v>0</v>
       </c>
-      <c r="M17" t="s">
-        <v>26</v>
-      </c>
-      <c r="N17" t="s">
-        <v>26</v>
-      </c>
-      <c r="O17" t="s">
-        <v>26</v>
-      </c>
-      <c r="P17" t="s">
-        <v>26</v>
+      <c r="Q17" t="s">
+        <v>32</v>
+      </c>
+      <c r="R17" t="s">
+        <v>32</v>
+      </c>
+      <c r="S17" t="s">
+        <v>32</v>
+      </c>
+      <c r="T17" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="B18" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="C18" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="E18" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F18" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G18" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="H18" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I18" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J18" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K18" t="s">
-        <v>26</v>
-      </c>
-      <c r="L18" t="b">
+        <v>32</v>
+      </c>
+      <c r="L18" t="s">
+        <v>32</v>
+      </c>
+      <c r="M18" t="s">
+        <v>32</v>
+      </c>
+      <c r="N18" t="s">
+        <v>32</v>
+      </c>
+      <c r="O18" t="s">
+        <v>32</v>
+      </c>
+      <c r="P18" t="b">
         <v>0</v>
       </c>
-      <c r="M18" t="s">
-        <v>26</v>
-      </c>
-      <c r="N18" t="s">
-        <v>26</v>
-      </c>
-      <c r="O18" t="s">
-        <v>26</v>
-      </c>
-      <c r="P18" t="s">
-        <v>26</v>
+      <c r="Q18" t="s">
+        <v>32</v>
+      </c>
+      <c r="R18" t="s">
+        <v>32</v>
+      </c>
+      <c r="S18" t="s">
+        <v>32</v>
+      </c>
+      <c r="T18" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="B19" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="C19" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D19" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="E19" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F19" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G19" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H19" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I19" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J19" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K19" t="s">
-        <v>26</v>
-      </c>
-      <c r="L19" t="b">
+        <v>32</v>
+      </c>
+      <c r="L19" t="s">
+        <v>32</v>
+      </c>
+      <c r="M19" t="s">
+        <v>32</v>
+      </c>
+      <c r="N19" t="s">
+        <v>32</v>
+      </c>
+      <c r="O19" t="s">
+        <v>32</v>
+      </c>
+      <c r="P19" t="b">
         <v>0</v>
       </c>
-      <c r="M19" t="s">
-        <v>26</v>
-      </c>
-      <c r="N19" t="s">
-        <v>26</v>
-      </c>
-      <c r="O19" t="s">
-        <v>26</v>
-      </c>
-      <c r="P19" t="s">
-        <v>26</v>
+      <c r="Q19" t="s">
+        <v>32</v>
+      </c>
+      <c r="R19" t="s">
+        <v>32</v>
+      </c>
+      <c r="S19" t="s">
+        <v>32</v>
+      </c>
+      <c r="T19" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -2423,82 +2901,82 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="10.71875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="12.203125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="13.6171875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -2515,59 +2993,59 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="10.23828125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="11.94140625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="13.6171875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
conf scheduling: add audience level and content tags + change speakers column order
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -13,12 +13,13 @@
     <sheet name="Talks" r:id="rId7" sheetId="5"/>
     <sheet name="Theme view" r:id="rId8" sheetId="6"/>
     <sheet name="Sector view" r:id="rId9" sheetId="7"/>
+    <sheet name="Speaker view" r:id="rId10" sheetId="8"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="165">
   <si>
     <t>Conference name</t>
   </si>
@@ -173,271 +174,346 @@
     <t>Large, Recorded</t>
   </si>
   <si>
+    <t>S06</t>
+  </si>
+  <si>
+    <t>R 2</t>
+  </si>
+  <si>
+    <t>R 3</t>
+  </si>
+  <si>
+    <t>Recorded</t>
+  </si>
+  <si>
+    <t>R 4</t>
+  </si>
+  <si>
+    <t>R 5</t>
+  </si>
+  <si>
+    <t>Lab_room, Large, Recorded</t>
+  </si>
+  <si>
+    <t>Required timeslot tags</t>
+  </si>
+  <si>
+    <t>Preferred timeslot tags</t>
+  </si>
+  <si>
+    <t>Prohibited timeslot tags</t>
+  </si>
+  <si>
+    <t>Undesired timeslot tags</t>
+  </si>
+  <si>
+    <t>Required room tags</t>
+  </si>
+  <si>
+    <t>Preferred room tags</t>
+  </si>
+  <si>
+    <t>Prohibited room tags</t>
+  </si>
+  <si>
+    <t>Undesired room tags</t>
+  </si>
+  <si>
+    <t>Amy Cole</t>
+  </si>
+  <si>
+    <t>Beth Fox</t>
+  </si>
+  <si>
+    <t>Chad Green</t>
+  </si>
+  <si>
+    <t>Dan Jones</t>
+  </si>
+  <si>
+    <t>Elsa King</t>
+  </si>
+  <si>
+    <t>Flo Li</t>
+  </si>
+  <si>
+    <t>Gus Poe</t>
+  </si>
+  <si>
+    <t>Hugo Rye</t>
+  </si>
+  <si>
+    <t>Ivy Smith</t>
+  </si>
+  <si>
+    <t>Jay Watt</t>
+  </si>
+  <si>
+    <t>Amy Fox</t>
+  </si>
+  <si>
+    <t>Beth Green</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Speakers</t>
+  </si>
+  <si>
+    <t>Theme tags</t>
+  </si>
+  <si>
+    <t>Sector tags</t>
+  </si>
+  <si>
+    <t>Audience level</t>
+  </si>
+  <si>
+    <t>Content tags</t>
+  </si>
+  <si>
+    <t>Language</t>
+  </si>
+  <si>
+    <t>Pinned by user</t>
+  </si>
+  <si>
+    <t>Timeslot day</t>
+  </si>
+  <si>
+    <t>Room</t>
+  </si>
+  <si>
+    <t>S00</t>
+  </si>
+  <si>
+    <t>Hands on real-time OpenShift</t>
+  </si>
+  <si>
+    <t>Cloud</t>
+  </si>
+  <si>
+    <t>Government</t>
+  </si>
+  <si>
+    <t>OpenShift, Kubernetes</t>
+  </si>
+  <si>
+    <t>en</t>
+  </si>
+  <si>
+    <t>Lab_room</t>
+  </si>
+  <si>
+    <t>S01</t>
+  </si>
+  <si>
+    <t>Advanced containerized WildFly</t>
+  </si>
+  <si>
+    <t>Big Data</t>
+  </si>
+  <si>
+    <t>WildFly</t>
+  </si>
+  <si>
+    <t>S02</t>
+  </si>
+  <si>
+    <t>Learn virtualized Spring</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>Spring</t>
+  </si>
+  <si>
+    <t>S03</t>
+  </si>
+  <si>
+    <t>Intro to serverless Drools</t>
+  </si>
+  <si>
+    <t>Culture</t>
+  </si>
+  <si>
+    <t>Drools</t>
+  </si>
+  <si>
+    <t>S04</t>
+  </si>
+  <si>
+    <t>Discover AI-driven OptaPlanner</t>
+  </si>
+  <si>
+    <t>Elsa King, Flo Li</t>
+  </si>
+  <si>
+    <t>IoT</t>
+  </si>
+  <si>
+    <t>OptaPlanner</t>
+  </si>
+  <si>
     <t>S05</t>
   </si>
   <si>
-    <t>R 2</t>
-  </si>
-  <si>
-    <t>R 3</t>
-  </si>
-  <si>
-    <t>Recorded</t>
-  </si>
-  <si>
-    <t>R 4</t>
-  </si>
-  <si>
-    <t>R 5</t>
-  </si>
-  <si>
-    <t>Lab_room, Large, Recorded</t>
-  </si>
-  <si>
-    <t>Required timeslot tags</t>
-  </si>
-  <si>
-    <t>Preferred timeslot tags</t>
-  </si>
-  <si>
-    <t>Prohibited timeslot tags</t>
-  </si>
-  <si>
-    <t>Undesired timeslot tags</t>
-  </si>
-  <si>
-    <t>Required room tags</t>
-  </si>
-  <si>
-    <t>Preferred room tags</t>
-  </si>
-  <si>
-    <t>Prohibited room tags</t>
-  </si>
-  <si>
-    <t>Undesired room tags</t>
-  </si>
-  <si>
-    <t>Amy Cole</t>
-  </si>
-  <si>
-    <t>Beth Fox</t>
-  </si>
-  <si>
-    <t>Chad Green</t>
-  </si>
-  <si>
-    <t>Dan Jones</t>
-  </si>
-  <si>
-    <t>Elsa King</t>
-  </si>
-  <si>
-    <t>Flo Li</t>
-  </si>
-  <si>
-    <t>Gus Poe</t>
-  </si>
-  <si>
-    <t>Hugo Rye</t>
-  </si>
-  <si>
-    <t>Ivy Smith</t>
-  </si>
-  <si>
-    <t>Jay Watt</t>
-  </si>
-  <si>
-    <t>Amy Fox</t>
-  </si>
-  <si>
-    <t>Beth Green</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>Theme tags</t>
-  </si>
-  <si>
-    <t>Sector tags</t>
-  </si>
-  <si>
-    <t>Language</t>
-  </si>
-  <si>
-    <t>Speakers</t>
-  </si>
-  <si>
-    <t>Pinned by user</t>
-  </si>
-  <si>
-    <t>Timeslot day</t>
-  </si>
-  <si>
-    <t>Room</t>
-  </si>
-  <si>
-    <t>S00</t>
-  </si>
-  <si>
-    <t>Hands on real-time OpenShift</t>
-  </si>
-  <si>
-    <t>Mobile</t>
-  </si>
-  <si>
-    <t>en</t>
+    <t>Mastering machine learning jBPM</t>
+  </si>
+  <si>
+    <t>Gus Poe, Hugo Rye</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>jBPM</t>
+  </si>
+  <si>
+    <t>Tuning IOT-driven Camel</t>
+  </si>
+  <si>
+    <t>Artificial Intelligence</t>
+  </si>
+  <si>
+    <t>Camel</t>
+  </si>
+  <si>
+    <t>S07</t>
+  </si>
+  <si>
+    <t>Building deep learning XStream</t>
+  </si>
+  <si>
+    <t>XStream</t>
+  </si>
+  <si>
+    <t>S08</t>
+  </si>
+  <si>
+    <t>Securing scalable Docker</t>
+  </si>
+  <si>
+    <t>Amy Fox, Beth Green</t>
+  </si>
+  <si>
+    <t>Modern Web</t>
+  </si>
+  <si>
+    <t>Docker</t>
+  </si>
+  <si>
+    <t>S09</t>
+  </si>
+  <si>
+    <t>Debug enterprise Hibernate</t>
+  </si>
+  <si>
+    <t>Hibernate</t>
+  </si>
+  <si>
+    <t>S10</t>
+  </si>
+  <si>
+    <t>Prepare for streaming GWT</t>
+  </si>
+  <si>
+    <t>Beth Fox, Chad Green</t>
+  </si>
+  <si>
+    <t>Security, Cloud</t>
+  </si>
+  <si>
+    <t>GWT</t>
+  </si>
+  <si>
+    <t>S11</t>
+  </si>
+  <si>
+    <t>Understand mobile Errai</t>
+  </si>
+  <si>
+    <t>Errai</t>
+  </si>
+  <si>
+    <t>S12</t>
+  </si>
+  <si>
+    <t>Applying modern Angular</t>
+  </si>
+  <si>
+    <t>Angular</t>
+  </si>
+  <si>
+    <t>S13</t>
+  </si>
+  <si>
+    <t>Grok distributed Weld</t>
+  </si>
+  <si>
+    <t>Weld</t>
+  </si>
+  <si>
+    <t>S14</t>
+  </si>
+  <si>
+    <t>Troubleshooting reliable RestEasy</t>
+  </si>
+  <si>
+    <t>Security, Mobile</t>
+  </si>
+  <si>
+    <t>RestEasy</t>
+  </si>
+  <si>
+    <t>S15</t>
+  </si>
+  <si>
+    <t>Using secure Android</t>
+  </si>
+  <si>
+    <t>Android</t>
+  </si>
+  <si>
+    <t>S16</t>
+  </si>
+  <si>
+    <t>Deliver stable Tensorflow</t>
+  </si>
+  <si>
+    <t>Cloud, Modern Web</t>
+  </si>
+  <si>
+    <t>Tensorflow</t>
+  </si>
+  <si>
+    <t>S17</t>
+  </si>
+  <si>
+    <t>Implement platform-independent VertX</t>
   </si>
   <si>
     <t>Amy Cole, Beth Fox</t>
   </si>
   <si>
-    <t>Lab_room</t>
-  </si>
-  <si>
-    <t>S01</t>
-  </si>
-  <si>
-    <t>Advanced containerized WildFly</t>
-  </si>
-  <si>
-    <t>Big Data</t>
-  </si>
-  <si>
-    <t>S02</t>
-  </si>
-  <si>
-    <t>Learn virtualized Spring</t>
-  </si>
-  <si>
-    <t>Artificial Intelligence</t>
-  </si>
-  <si>
-    <t>Transportation</t>
-  </si>
-  <si>
-    <t>Dan Jones, Elsa King</t>
-  </si>
-  <si>
-    <t>S03</t>
-  </si>
-  <si>
-    <t>Intro to serverless Drools</t>
-  </si>
-  <si>
-    <t>Mobile, Big Data</t>
-  </si>
-  <si>
-    <t>S04</t>
-  </si>
-  <si>
-    <t>Discover AI-driven OptaPlanner</t>
-  </si>
-  <si>
-    <t>Cloud</t>
-  </si>
-  <si>
-    <t>Mastering machine learning jBPM</t>
-  </si>
-  <si>
-    <t>Hugo Rye, Ivy Smith</t>
-  </si>
-  <si>
-    <t>S06</t>
-  </si>
-  <si>
-    <t>Tuning IOT-driven Camel</t>
-  </si>
-  <si>
-    <t>Security</t>
-  </si>
-  <si>
-    <t>Jay Watt, Amy Fox</t>
-  </si>
-  <si>
-    <t>S07</t>
-  </si>
-  <si>
-    <t>Building deep learning XStream</t>
-  </si>
-  <si>
-    <t>S08</t>
-  </si>
-  <si>
-    <t>Securing scalable Docker</t>
-  </si>
-  <si>
-    <t>IoT</t>
-  </si>
-  <si>
-    <t>S09</t>
-  </si>
-  <si>
-    <t>Debug enterprise JUnit</t>
-  </si>
-  <si>
-    <t>Culture, Security</t>
-  </si>
-  <si>
-    <t>S10</t>
-  </si>
-  <si>
-    <t>Hands on real-time WildFly</t>
-  </si>
-  <si>
-    <t>S11</t>
-  </si>
-  <si>
-    <t>Advanced containerized Spring</t>
-  </si>
-  <si>
-    <t>S12</t>
-  </si>
-  <si>
-    <t>Learn virtualized Drools</t>
-  </si>
-  <si>
-    <t>S13</t>
-  </si>
-  <si>
-    <t>Intro to serverless OptaPlanner</t>
-  </si>
-  <si>
-    <t>S14</t>
-  </si>
-  <si>
-    <t>Discover AI-driven jBPM</t>
-  </si>
-  <si>
-    <t>S15</t>
-  </si>
-  <si>
-    <t>Mastering machine learning Camel</t>
-  </si>
-  <si>
-    <t>Mobile, Security</t>
-  </si>
-  <si>
-    <t>S16</t>
-  </si>
-  <si>
-    <t>Tuning IOT-driven XStream</t>
-  </si>
-  <si>
-    <t>S17</t>
-  </si>
-  <si>
-    <t>Building deep learning Docker</t>
+    <t>Middleware, Modern Web</t>
+  </si>
+  <si>
+    <t>VertX</t>
   </si>
   <si>
     <t>Theme tag</t>
   </si>
   <si>
     <t>Sector tag</t>
+  </si>
+  <si>
+    <t>Speaker</t>
   </si>
 </sst>
 </file>
@@ -459,7 +535,7 @@
       <b val="true"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -479,6 +555,16 @@
         <fgColor rgb="AD7FA8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="EF2929"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FCAF3E"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -492,11 +578,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -506,9 +594,9 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="33.8671875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="12.33203125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="81.296875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="29.5" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="11.80859375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="70.88671875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -662,11 +750,11 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="16.14453125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="6.3984375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="6.32421875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="10.78515625" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="6.078125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="15.99609375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="6.0859375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="6.0859375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="9.41796875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="5.1484375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -798,14 +886,14 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="7.109375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="26.3125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="6.48828125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="25.6328125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="11.86328125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1003,21 +1091,21 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="11.9453125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="24.85546875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="25.390625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="26.30859375" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="26.0234375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="21.671875" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="22.20703125" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="23.125" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="22.84375" customWidth="true" bestFit="true"/>
-    <col min="10" max="10" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="12" max="12" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="13" max="13" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="14" max="14" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="15" max="15" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="11.5703125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="21.69921875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="22.09765625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="23.01171875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="22.7734375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="19.07421875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="19.47265625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="20.3828125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="20.1484375" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="14" max="14" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" width="11.86328125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1475,7 +1563,7 @@
         <v>32</v>
       </c>
       <c r="K10" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="L10" t="s">
         <v>32</v>
@@ -1691,26 +1779,28 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="6.34765625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="33.1015625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.78515625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="19.83203125" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="14.55078125" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="11.3046875" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="19.76171875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="24.85546875" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="25.390625" customWidth="true" bestFit="true"/>
-    <col min="10" max="10" width="26.30859375" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="26.0234375" customWidth="true" bestFit="true"/>
-    <col min="12" max="12" width="21.671875" customWidth="true" bestFit="true"/>
-    <col min="13" max="13" width="22.20703125" customWidth="true" bestFit="true"/>
-    <col min="14" max="14" width="23.125" customWidth="true" bestFit="true"/>
-    <col min="15" max="15" width="22.84375" customWidth="true" bestFit="true"/>
-    <col min="16" max="16" width="16.65234375" customWidth="true" bestFit="true"/>
-    <col min="17" max="17" width="16.14453125" customWidth="true" bestFit="true"/>
-    <col min="18" max="18" width="6.3984375" customWidth="true" bestFit="true"/>
-    <col min="19" max="19" width="6.32421875" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="7.02734375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="5.69140625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="36.7734375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="9.41796875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="20.421875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="24.78515625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="12.33984375" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="14.4375" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="21.28515625" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="9.7109375" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="21.69921875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="22.09765625" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" width="23.01171875" customWidth="true" bestFit="true"/>
+    <col min="13" max="13" width="22.7734375" customWidth="true" bestFit="true"/>
+    <col min="14" max="14" width="19.07421875" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" width="19.47265625" customWidth="true" bestFit="true"/>
+    <col min="16" max="16" width="20.3828125" customWidth="true" bestFit="true"/>
+    <col min="17" max="17" width="20.1484375" customWidth="true" bestFit="true"/>
+    <col min="18" max="18" width="14.578125" customWidth="true" bestFit="true"/>
+    <col min="19" max="19" width="15.99609375" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="6.0859375" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="6.0859375" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="6.44921875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1736,72 +1826,78 @@
         <v>83</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="P1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="R1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="T1" s="1" t="s">
-        <v>86</v>
+      <c r="V1" s="1" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C2" t="s">
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="E2" t="s">
-        <v>32</v>
+        <v>91</v>
       </c>
       <c r="F2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G2" t="s">
-        <v>91</v>
+        <v>92</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2.0</v>
       </c>
       <c r="H2" t="s">
-        <v>32</v>
+        <v>93</v>
       </c>
       <c r="I2" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J2" t="s">
         <v>32</v>
@@ -1810,122 +1906,134 @@
         <v>32</v>
       </c>
       <c r="L2" t="s">
-        <v>92</v>
+        <v>32</v>
       </c>
       <c r="M2" t="s">
         <v>32</v>
       </c>
       <c r="N2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="O2" t="s">
         <v>32</v>
       </c>
-      <c r="P2" t="b">
+      <c r="P2" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>32</v>
+      </c>
+      <c r="R2" t="b">
         <v>0</v>
       </c>
-      <c r="Q2" t="s">
-        <v>32</v>
-      </c>
-      <c r="R2" t="s">
-        <v>32</v>
-      </c>
       <c r="S2" t="s">
         <v>32</v>
       </c>
       <c r="T2" t="s">
+        <v>32</v>
+      </c>
+      <c r="U2" t="s">
+        <v>32</v>
+      </c>
+      <c r="V2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
         <v>31</v>
       </c>
       <c r="D3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>99</v>
+      </c>
+      <c r="I3" t="s">
+        <v>94</v>
+      </c>
+      <c r="J3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M3" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3" t="s">
         <v>95</v>
       </c>
-      <c r="E3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F3" t="s">
-        <v>90</v>
-      </c>
-      <c r="G3" t="s">
-        <v>68</v>
-      </c>
-      <c r="H3" t="s">
-        <v>32</v>
-      </c>
-      <c r="I3" t="s">
-        <v>32</v>
-      </c>
-      <c r="J3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K3" t="s">
-        <v>32</v>
-      </c>
-      <c r="L3" t="s">
-        <v>92</v>
-      </c>
-      <c r="M3" t="s">
-        <v>32</v>
-      </c>
-      <c r="N3" t="s">
-        <v>32</v>
-      </c>
       <c r="O3" t="s">
         <v>32</v>
       </c>
-      <c r="P3" t="b">
+      <c r="P3" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>32</v>
+      </c>
+      <c r="R3" t="b">
         <v>0</v>
       </c>
-      <c r="Q3" t="s">
-        <v>32</v>
-      </c>
-      <c r="R3" t="s">
-        <v>32</v>
-      </c>
       <c r="S3" t="s">
         <v>32</v>
       </c>
       <c r="T3" t="s">
+        <v>32</v>
+      </c>
+      <c r="U3" t="s">
+        <v>32</v>
+      </c>
+      <c r="V3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B4" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C4" t="s">
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="E4" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="F4" t="s">
-        <v>90</v>
-      </c>
-      <c r="G4" t="s">
-        <v>100</v>
+        <v>32</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3.0</v>
       </c>
       <c r="H4" t="s">
-        <v>32</v>
+        <v>103</v>
       </c>
       <c r="I4" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J4" t="s">
         <v>32</v>
@@ -1945,49 +2053,55 @@
       <c r="O4" t="s">
         <v>32</v>
       </c>
-      <c r="P4" t="b">
+      <c r="P4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>32</v>
+      </c>
+      <c r="R4" t="b">
         <v>0</v>
       </c>
-      <c r="Q4" t="s">
-        <v>32</v>
-      </c>
-      <c r="R4" t="s">
-        <v>32</v>
-      </c>
       <c r="S4" t="s">
         <v>32</v>
       </c>
       <c r="T4" t="s">
+        <v>32</v>
+      </c>
+      <c r="U4" t="s">
+        <v>32</v>
+      </c>
+      <c r="V4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C5" t="s">
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
       <c r="E5" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="F5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G5" t="s">
-        <v>71</v>
+        <v>32</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2.0</v>
       </c>
       <c r="H5" t="s">
-        <v>32</v>
+        <v>107</v>
       </c>
       <c r="I5" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J5" t="s">
         <v>32</v>
@@ -2007,49 +2121,55 @@
       <c r="O5" t="s">
         <v>32</v>
       </c>
-      <c r="P5" t="b">
+      <c r="P5" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>32</v>
+      </c>
+      <c r="R5" t="b">
         <v>0</v>
       </c>
-      <c r="Q5" t="s">
-        <v>32</v>
-      </c>
-      <c r="R5" t="s">
-        <v>32</v>
-      </c>
       <c r="S5" t="s">
         <v>32</v>
       </c>
       <c r="T5" t="s">
+        <v>32</v>
+      </c>
+      <c r="U5" t="s">
+        <v>32</v>
+      </c>
+      <c r="V5" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B6" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C6" t="s">
         <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>111</v>
       </c>
       <c r="F6" t="s">
-        <v>90</v>
-      </c>
-      <c r="G6" t="s">
-        <v>72</v>
+        <v>32</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3.0</v>
       </c>
       <c r="H6" t="s">
-        <v>32</v>
+        <v>112</v>
       </c>
       <c r="I6" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J6" t="s">
         <v>32</v>
@@ -2069,49 +2189,55 @@
       <c r="O6" t="s">
         <v>32</v>
       </c>
-      <c r="P6" t="b">
+      <c r="P6" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>32</v>
+      </c>
+      <c r="R6" t="b">
         <v>0</v>
       </c>
-      <c r="Q6" t="s">
-        <v>32</v>
-      </c>
-      <c r="R6" t="s">
-        <v>32</v>
-      </c>
       <c r="S6" t="s">
         <v>32</v>
       </c>
       <c r="T6" t="s">
+        <v>32</v>
+      </c>
+      <c r="U6" t="s">
+        <v>32</v>
+      </c>
+      <c r="V6" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>113</v>
       </c>
       <c r="B7" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="C7" t="s">
         <v>34</v>
       </c>
       <c r="D7" t="s">
-        <v>89</v>
+        <v>115</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>116</v>
       </c>
       <c r="F7" t="s">
-        <v>90</v>
-      </c>
-      <c r="G7" t="s">
-        <v>108</v>
+        <v>32</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.0</v>
       </c>
       <c r="H7" t="s">
-        <v>32</v>
+        <v>117</v>
       </c>
       <c r="I7" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J7" t="s">
         <v>32</v>
@@ -2131,49 +2257,55 @@
       <c r="O7" t="s">
         <v>32</v>
       </c>
-      <c r="P7" s="3" t="b">
-        <v>1</v>
+      <c r="P7" t="s">
+        <v>32</v>
       </c>
       <c r="Q7" t="s">
-        <v>28</v>
-      </c>
-      <c r="R7" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="R7" t="b">
+        <v>0</v>
       </c>
       <c r="S7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="T7" t="s">
-        <v>49</v>
+        <v>32</v>
+      </c>
+      <c r="U7" t="s">
+        <v>32</v>
+      </c>
+      <c r="V7" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>109</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="C8" t="s">
         <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>111</v>
+        <v>74</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>119</v>
       </c>
       <c r="F8" t="s">
-        <v>90</v>
-      </c>
-      <c r="G8" t="s">
-        <v>112</v>
+        <v>32</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.0</v>
       </c>
       <c r="H8" t="s">
-        <v>32</v>
+        <v>120</v>
       </c>
       <c r="I8" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J8" t="s">
         <v>32</v>
@@ -2193,49 +2325,55 @@
       <c r="O8" t="s">
         <v>32</v>
       </c>
-      <c r="P8" t="b">
-        <v>0</v>
+      <c r="P8" t="s">
+        <v>32</v>
       </c>
       <c r="Q8" t="s">
         <v>32</v>
       </c>
-      <c r="R8" t="s">
-        <v>32</v>
+      <c r="R8" s="3" t="b">
+        <v>1</v>
       </c>
       <c r="S8" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="T8" t="s">
-        <v>32</v>
+        <v>29</v>
+      </c>
+      <c r="U8" t="s">
+        <v>33</v>
+      </c>
+      <c r="V8" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="B9" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C9" t="s">
         <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>111</v>
       </c>
       <c r="F9" t="s">
-        <v>90</v>
-      </c>
-      <c r="G9" t="s">
-        <v>77</v>
+        <v>32</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2.0</v>
       </c>
       <c r="H9" t="s">
-        <v>32</v>
+        <v>123</v>
       </c>
       <c r="I9" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J9" t="s">
         <v>32</v>
@@ -2255,49 +2393,55 @@
       <c r="O9" t="s">
         <v>32</v>
       </c>
-      <c r="P9" t="b">
+      <c r="P9" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>32</v>
+      </c>
+      <c r="R9" t="b">
         <v>0</v>
       </c>
-      <c r="Q9" t="s">
-        <v>32</v>
-      </c>
-      <c r="R9" t="s">
-        <v>32</v>
-      </c>
       <c r="S9" t="s">
         <v>32</v>
       </c>
       <c r="T9" t="s">
+        <v>32</v>
+      </c>
+      <c r="U9" t="s">
+        <v>32</v>
+      </c>
+      <c r="V9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="B10" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="C10" t="s">
         <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="E10" t="s">
-        <v>32</v>
+        <v>127</v>
       </c>
       <c r="F10" t="s">
-        <v>90</v>
-      </c>
-      <c r="G10" t="s">
-        <v>91</v>
+        <v>32</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3.0</v>
       </c>
       <c r="H10" t="s">
-        <v>32</v>
+        <v>128</v>
       </c>
       <c r="I10" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J10" t="s">
         <v>32</v>
@@ -2317,49 +2461,55 @@
       <c r="O10" t="s">
         <v>32</v>
       </c>
-      <c r="P10" t="b">
+      <c r="P10" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>32</v>
+      </c>
+      <c r="R10" t="b">
         <v>0</v>
       </c>
-      <c r="Q10" t="s">
-        <v>32</v>
-      </c>
-      <c r="R10" t="s">
-        <v>32</v>
-      </c>
       <c r="S10" t="s">
         <v>32</v>
       </c>
       <c r="T10" t="s">
+        <v>32</v>
+      </c>
+      <c r="U10" t="s">
+        <v>32</v>
+      </c>
+      <c r="V10" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="B11" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="C11" t="s">
         <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>120</v>
+        <v>66</v>
       </c>
       <c r="E11" t="s">
-        <v>32</v>
+        <v>119</v>
       </c>
       <c r="F11" t="s">
-        <v>90</v>
-      </c>
-      <c r="G11" t="s">
-        <v>68</v>
+        <v>32</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.0</v>
       </c>
       <c r="H11" t="s">
-        <v>32</v>
+        <v>131</v>
       </c>
       <c r="I11" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J11" t="s">
         <v>32</v>
@@ -2379,49 +2529,55 @@
       <c r="O11" t="s">
         <v>32</v>
       </c>
-      <c r="P11" t="b">
+      <c r="P11" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>32</v>
+      </c>
+      <c r="R11" t="b">
         <v>0</v>
       </c>
-      <c r="Q11" t="s">
-        <v>32</v>
-      </c>
-      <c r="R11" t="s">
-        <v>32</v>
-      </c>
       <c r="S11" t="s">
         <v>32</v>
       </c>
       <c r="T11" t="s">
+        <v>32</v>
+      </c>
+      <c r="U11" t="s">
+        <v>32</v>
+      </c>
+      <c r="V11" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="B12" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="C12" t="s">
         <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>89</v>
+        <v>134</v>
       </c>
       <c r="E12" t="s">
-        <v>32</v>
+        <v>135</v>
       </c>
       <c r="F12" t="s">
-        <v>90</v>
-      </c>
-      <c r="G12" t="s">
-        <v>69</v>
+        <v>32</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3.0</v>
       </c>
       <c r="H12" t="s">
-        <v>32</v>
+        <v>136</v>
       </c>
       <c r="I12" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J12" t="s">
         <v>32</v>
@@ -2441,49 +2597,55 @@
       <c r="O12" t="s">
         <v>32</v>
       </c>
-      <c r="P12" t="b">
+      <c r="P12" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>32</v>
+      </c>
+      <c r="R12" t="b">
         <v>0</v>
       </c>
-      <c r="Q12" t="s">
-        <v>32</v>
-      </c>
-      <c r="R12" t="s">
-        <v>32</v>
-      </c>
       <c r="S12" t="s">
         <v>32</v>
       </c>
       <c r="T12" t="s">
+        <v>32</v>
+      </c>
+      <c r="U12" t="s">
+        <v>32</v>
+      </c>
+      <c r="V12" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="B13" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="C13" t="s">
         <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>117</v>
+        <v>69</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
+        <v>111</v>
       </c>
       <c r="F13" t="s">
-        <v>90</v>
-      </c>
-      <c r="G13" t="s">
-        <v>70</v>
+        <v>32</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3.0</v>
       </c>
       <c r="H13" t="s">
-        <v>32</v>
+        <v>139</v>
       </c>
       <c r="I13" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J13" t="s">
         <v>32</v>
@@ -2503,49 +2665,55 @@
       <c r="O13" t="s">
         <v>32</v>
       </c>
-      <c r="P13" t="b">
+      <c r="P13" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>32</v>
+      </c>
+      <c r="R13" t="b">
         <v>0</v>
       </c>
-      <c r="Q13" t="s">
-        <v>32</v>
-      </c>
-      <c r="R13" t="s">
-        <v>32</v>
-      </c>
       <c r="S13" t="s">
         <v>32</v>
       </c>
       <c r="T13" t="s">
+        <v>32</v>
+      </c>
+      <c r="U13" t="s">
+        <v>32</v>
+      </c>
+      <c r="V13" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="B14" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="C14" t="s">
         <v>34</v>
       </c>
       <c r="D14" t="s">
+        <v>110</v>
+      </c>
+      <c r="E14" t="s">
         <v>106</v>
       </c>
-      <c r="E14" t="s">
-        <v>32</v>
-      </c>
       <c r="F14" t="s">
-        <v>90</v>
-      </c>
-      <c r="G14" t="s">
-        <v>71</v>
+        <v>32</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3.0</v>
       </c>
       <c r="H14" t="s">
-        <v>32</v>
+        <v>142</v>
       </c>
       <c r="I14" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J14" t="s">
         <v>32</v>
@@ -2565,49 +2733,55 @@
       <c r="O14" t="s">
         <v>32</v>
       </c>
-      <c r="P14" t="b">
+      <c r="P14" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>32</v>
+      </c>
+      <c r="R14" t="b">
         <v>0</v>
       </c>
-      <c r="Q14" t="s">
-        <v>32</v>
-      </c>
-      <c r="R14" t="s">
-        <v>32</v>
-      </c>
       <c r="S14" t="s">
         <v>32</v>
       </c>
       <c r="T14" t="s">
+        <v>32</v>
+      </c>
+      <c r="U14" t="s">
+        <v>32</v>
+      </c>
+      <c r="V14" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="B15" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="C15" t="s">
         <v>34</v>
       </c>
       <c r="D15" t="s">
-        <v>89</v>
+        <v>115</v>
       </c>
       <c r="E15" t="s">
-        <v>32</v>
+        <v>116</v>
       </c>
       <c r="F15" t="s">
-        <v>90</v>
-      </c>
-      <c r="G15" t="s">
-        <v>72</v>
+        <v>32</v>
+      </c>
+      <c r="G15" t="n">
+        <v>3.0</v>
       </c>
       <c r="H15" t="s">
-        <v>32</v>
+        <v>145</v>
       </c>
       <c r="I15" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J15" t="s">
         <v>32</v>
@@ -2627,49 +2801,55 @@
       <c r="O15" t="s">
         <v>32</v>
       </c>
-      <c r="P15" t="b">
+      <c r="P15" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>32</v>
+      </c>
+      <c r="R15" t="b">
         <v>0</v>
       </c>
-      <c r="Q15" t="s">
-        <v>32</v>
-      </c>
-      <c r="R15" t="s">
-        <v>32</v>
-      </c>
       <c r="S15" t="s">
         <v>32</v>
       </c>
       <c r="T15" t="s">
+        <v>32</v>
+      </c>
+      <c r="U15" t="s">
+        <v>32</v>
+      </c>
+      <c r="V15" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="B16" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="C16" t="s">
         <v>34</v>
       </c>
       <c r="D16" t="s">
-        <v>111</v>
+        <v>74</v>
       </c>
       <c r="E16" t="s">
-        <v>32</v>
+        <v>148</v>
       </c>
       <c r="F16" t="s">
-        <v>90</v>
-      </c>
-      <c r="G16" t="s">
-        <v>108</v>
+        <v>32</v>
+      </c>
+      <c r="G16" t="n">
+        <v>3.0</v>
       </c>
       <c r="H16" t="s">
-        <v>32</v>
+        <v>149</v>
       </c>
       <c r="I16" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J16" t="s">
         <v>32</v>
@@ -2689,49 +2869,55 @@
       <c r="O16" t="s">
         <v>32</v>
       </c>
-      <c r="P16" t="b">
+      <c r="P16" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>32</v>
+      </c>
+      <c r="R16" t="b">
         <v>0</v>
       </c>
-      <c r="Q16" t="s">
-        <v>32</v>
-      </c>
-      <c r="R16" t="s">
-        <v>32</v>
-      </c>
       <c r="S16" t="s">
         <v>32</v>
       </c>
       <c r="T16" t="s">
+        <v>32</v>
+      </c>
+      <c r="U16" t="s">
+        <v>32</v>
+      </c>
+      <c r="V16" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="B17" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="C17" t="s">
         <v>34</v>
       </c>
       <c r="D17" t="s">
-        <v>133</v>
+        <v>75</v>
       </c>
       <c r="E17" t="s">
-        <v>32</v>
+        <v>98</v>
       </c>
       <c r="F17" t="s">
-        <v>90</v>
-      </c>
-      <c r="G17" t="s">
-        <v>112</v>
+        <v>32</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1.0</v>
       </c>
       <c r="H17" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="I17" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J17" t="s">
         <v>32</v>
@@ -2751,49 +2937,55 @@
       <c r="O17" t="s">
         <v>32</v>
       </c>
-      <c r="P17" t="b">
+      <c r="P17" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>32</v>
+      </c>
+      <c r="R17" t="b">
         <v>0</v>
       </c>
-      <c r="Q17" t="s">
-        <v>32</v>
-      </c>
-      <c r="R17" t="s">
-        <v>32</v>
-      </c>
       <c r="S17" t="s">
         <v>32</v>
       </c>
       <c r="T17" t="s">
+        <v>32</v>
+      </c>
+      <c r="U17" t="s">
+        <v>32</v>
+      </c>
+      <c r="V17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>134</v>
+        <v>153</v>
       </c>
       <c r="B18" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="C18" t="s">
         <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="E18" t="s">
-        <v>32</v>
+        <v>155</v>
       </c>
       <c r="F18" t="s">
-        <v>90</v>
-      </c>
-      <c r="G18" t="s">
-        <v>77</v>
+        <v>32</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2.0</v>
       </c>
       <c r="H18" t="s">
-        <v>32</v>
+        <v>156</v>
       </c>
       <c r="I18" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J18" t="s">
         <v>32</v>
@@ -2813,49 +3005,55 @@
       <c r="O18" t="s">
         <v>32</v>
       </c>
-      <c r="P18" t="b">
+      <c r="P18" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>32</v>
+      </c>
+      <c r="R18" t="b">
         <v>0</v>
       </c>
-      <c r="Q18" t="s">
-        <v>32</v>
-      </c>
-      <c r="R18" t="s">
-        <v>32</v>
-      </c>
       <c r="S18" t="s">
         <v>32</v>
       </c>
       <c r="T18" t="s">
+        <v>32</v>
+      </c>
+      <c r="U18" t="s">
+        <v>32</v>
+      </c>
+      <c r="V18" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="B19" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="C19" t="s">
         <v>34</v>
       </c>
       <c r="D19" t="s">
-        <v>117</v>
+        <v>159</v>
       </c>
       <c r="E19" t="s">
-        <v>32</v>
+        <v>160</v>
       </c>
       <c r="F19" t="s">
-        <v>90</v>
-      </c>
-      <c r="G19" t="s">
-        <v>91</v>
+        <v>92</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1.0</v>
       </c>
       <c r="H19" t="s">
-        <v>32</v>
+        <v>161</v>
       </c>
       <c r="I19" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="J19" t="s">
         <v>32</v>
@@ -2875,19 +3073,25 @@
       <c r="O19" t="s">
         <v>32</v>
       </c>
-      <c r="P19" t="b">
+      <c r="P19" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>32</v>
+      </c>
+      <c r="R19" t="b">
         <v>0</v>
       </c>
-      <c r="Q19" t="s">
-        <v>32</v>
-      </c>
-      <c r="R19" t="s">
-        <v>32</v>
-      </c>
       <c r="S19" t="s">
         <v>32</v>
       </c>
       <c r="T19" t="s">
+        <v>32</v>
+      </c>
+      <c r="U19" t="s">
+        <v>32</v>
+      </c>
+      <c r="V19" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2901,13 +3105,13 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="12.203125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="19.91015625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2935,7 +3139,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>43</v>
@@ -2958,26 +3162,16 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="B3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B3"/>
+      <c r="C3" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G3" t="s">
-        <v>32</v>
-      </c>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+      <c r="G3"/>
     </row>
   </sheetData>
   <sheetProtection password="D4D4" sheet="true" scenarios="true" objects="true"/>
@@ -2993,13 +3187,13 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="11.94140625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="13.6171875" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="13.6171875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="10.23828125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3027,7 +3221,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>43</v>
@@ -3046,6 +3240,351 @@
       </c>
       <c r="G2" s="1" t="s">
         <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection password="D4D4" sheet="true" scenarios="true" objects="true"/>
+  <mergeCells>
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="11.5703125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" t="s">
+        <v>32</v>
+      </c>
+      <c r="G8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" t="s">
+        <v>32</v>
+      </c>
+      <c r="G12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" t="s">
+        <v>32</v>
+      </c>
+      <c r="G13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" t="s">
+        <v>32</v>
+      </c>
+      <c r="G14" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
conf scheduling: add room and content view
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView activeTab="2"/>
+    <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" r:id="rId3" sheetId="1"/>
@@ -11,15 +11,17 @@
     <sheet name="Rooms" r:id="rId5" sheetId="3"/>
     <sheet name="Speakers" r:id="rId6" sheetId="4"/>
     <sheet name="Talks" r:id="rId7" sheetId="5"/>
-    <sheet name="Theme view" r:id="rId8" sheetId="6"/>
-    <sheet name="Sector view" r:id="rId9" sheetId="7"/>
-    <sheet name="Speaker view" r:id="rId10" sheetId="8"/>
+    <sheet name="Room view" r:id="rId8" sheetId="6"/>
+    <sheet name="Speaker view" r:id="rId9" sheetId="7"/>
+    <sheet name="Theme view" r:id="rId10" sheetId="8"/>
+    <sheet name="Sector view" r:id="rId11" sheetId="9"/>
+    <sheet name="Content view" r:id="rId12" sheetId="10"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="903" uniqueCount="167">
   <si>
     <t>Conference name</t>
   </si>
@@ -507,13 +509,19 @@
     <t>VertX</t>
   </si>
   <si>
+    <t>Speaker</t>
+  </si>
+  <si>
     <t>Theme tag</t>
   </si>
   <si>
     <t>Sector tag</t>
   </si>
   <si>
-    <t>Speaker</t>
+    <t>Content tag</t>
+  </si>
+  <si>
+    <t>(1) S06</t>
   </si>
 </sst>
 </file>
@@ -745,6 +753,88 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="11.78515625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3"/>
+      <c r="C3" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3"/>
+      <c r="G3"/>
+    </row>
+  </sheetData>
+  <sheetProtection password="D4D4" sheet="true" scenarios="true" objects="true"/>
+  <mergeCells>
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
@@ -3105,6 +3195,535 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
+    <col min="1" max="1" width="6.44921875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection password="D4D4" sheet="true" scenarios="true" objects="true"/>
+  <mergeCells>
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="11.5703125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" t="s">
+        <v>32</v>
+      </c>
+      <c r="G8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" t="s">
+        <v>32</v>
+      </c>
+      <c r="G12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" t="s">
+        <v>32</v>
+      </c>
+      <c r="G13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" t="s">
+        <v>32</v>
+      </c>
+      <c r="G14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection password="D4D4" sheet="true" scenarios="true" objects="true"/>
+  <mergeCells>
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
     <col min="1" max="1" width="19.91015625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
@@ -3139,7 +3758,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>43</v>
@@ -3182,7 +3801,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
@@ -3221,7 +3840,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>43</v>
@@ -3240,351 +3859,6 @@
       </c>
       <c r="G2" s="1" t="s">
         <v>48</v>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection password="D4D4" sheet="true" scenarios="true" objects="true"/>
-  <mergeCells>
-    <mergeCell ref="B1:G1"/>
-  </mergeCells>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F4" t="s">
-        <v>32</v>
-      </c>
-      <c r="G4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>69</v>
-      </c>
-      <c r="B6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" t="s">
-        <v>32</v>
-      </c>
-      <c r="F6" t="s">
-        <v>32</v>
-      </c>
-      <c r="G6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>71</v>
-      </c>
-      <c r="B8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F8" t="s">
-        <v>32</v>
-      </c>
-      <c r="G8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>72</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" t="s">
-        <v>32</v>
-      </c>
-      <c r="F9" t="s">
-        <v>32</v>
-      </c>
-      <c r="G9" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>73</v>
-      </c>
-      <c r="B10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10" t="s">
-        <v>32</v>
-      </c>
-      <c r="F10" t="s">
-        <v>32</v>
-      </c>
-      <c r="G10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>74</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" t="s">
-        <v>32</v>
-      </c>
-      <c r="F11" t="s">
-        <v>32</v>
-      </c>
-      <c r="G11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>75</v>
-      </c>
-      <c r="B12" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12" t="s">
-        <v>32</v>
-      </c>
-      <c r="F12" t="s">
-        <v>32</v>
-      </c>
-      <c r="G12" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>76</v>
-      </c>
-      <c r="B13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F13" t="s">
-        <v>32</v>
-      </c>
-      <c r="G13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>77</v>
-      </c>
-      <c r="B14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" t="s">
-        <v>32</v>
-      </c>
-      <c r="E14" t="s">
-        <v>32</v>
-      </c>
-      <c r="F14" t="s">
-        <v>32</v>
-      </c>
-      <c r="G14" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
conf scheduling: add constraint "Content audience level flow violation" (thanks Stephan)
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -20,8 +20,40 @@
 </workbook>
 </file>
 
+<file path=xl/comments10.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+    <author>OptaPlanner</author>
+  </authors>
+  <commentList>
+    <comment ref="C3" authorId="1">
+      <text>
+        <t>Speaker unavailable timeslots (S06): -1hard</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+    <author>OptaPlanner</author>
+  </authors>
+  <commentList>
+    <comment ref="C3" authorId="1">
+      <text>
+        <t>Speaker unavailable timeslots (S06): -1hard</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="903" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="169">
   <si>
     <t>Conference name</t>
   </si>
@@ -48,6 +80,12 @@
   </si>
   <si>
     <t>Soft penalty per common sector of 2 talks that have an overlapping timeslot</t>
+  </si>
+  <si>
+    <t>Content audience level flow violation</t>
+  </si>
+  <si>
+    <t>Soft penalty per common content of 2 talks with a different audience level for which the easier talk isn't scheduled earlier than the other talk.</t>
   </si>
   <si>
     <t>Language diversity</t>
@@ -597,14 +635,54 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="29.5" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="35.140625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="11.80859375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="70.88671875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="130.52734375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -690,12 +768,12 @@
         <v>10.0</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B10" t="n">
         <v>10.0</v>
@@ -706,13 +784,13 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B11" t="n">
         <v>10.0</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12">
@@ -734,12 +812,12 @@
         <v>10.0</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B14" t="n">
         <v>10.0</v>
@@ -748,13 +826,25 @@
         <v>20</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -769,57 +859,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B3"/>
       <c r="C3" s="4" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -827,16 +917,17 @@
       <c r="G3"/>
     </row>
   </sheetData>
-  <sheetProtection password="D4D4" sheet="true" scenarios="true" objects="true"/>
   <mergeCells>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -849,130 +940,131 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -988,184 +1080,184 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1173,11 +1265,12 @@
     <mergeCell ref="C1:H1"/>
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -1200,660 +1293,660 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1861,11 +1954,12 @@
     <mergeCell ref="J1:O1"/>
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -1895,1303 +1989,1304 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="U1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G2" t="n">
         <v>2.0</v>
       </c>
       <c r="H2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="O2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R2" t="b">
         <v>0</v>
       </c>
       <c r="S2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G3" t="n">
         <v>1.0</v>
       </c>
       <c r="H3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="O3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R3" t="b">
         <v>0</v>
       </c>
       <c r="S3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G4" t="n">
         <v>3.0</v>
       </c>
       <c r="H4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R4" t="b">
         <v>0</v>
       </c>
       <c r="S4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G5" t="n">
         <v>2.0</v>
       </c>
       <c r="H5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R5" t="b">
         <v>0</v>
       </c>
       <c r="S5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G6" t="n">
         <v>3.0</v>
       </c>
       <c r="H6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R6" t="b">
         <v>0</v>
       </c>
       <c r="S6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G7" t="n">
         <v>1.0</v>
       </c>
       <c r="H7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="I7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R7" t="b">
         <v>0</v>
       </c>
       <c r="S7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G8" t="n">
         <v>1.0</v>
       </c>
       <c r="H8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R8" s="3" t="b">
         <v>1</v>
       </c>
       <c r="S8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="T8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="U8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="V8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B9" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G9" t="n">
         <v>2.0</v>
       </c>
       <c r="H9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R9" t="b">
         <v>0</v>
       </c>
       <c r="S9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G10" t="n">
         <v>3.0</v>
       </c>
       <c r="H10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R10" t="b">
         <v>0</v>
       </c>
       <c r="S10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B11" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E11" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G11" t="n">
         <v>1.0</v>
       </c>
       <c r="H11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="I11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R11" t="b">
         <v>0</v>
       </c>
       <c r="S11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B12" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G12" t="n">
         <v>3.0</v>
       </c>
       <c r="H12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I12" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R12" t="b">
         <v>0</v>
       </c>
       <c r="S12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B13" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E13" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G13" t="n">
         <v>3.0</v>
       </c>
       <c r="H13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R13" t="b">
         <v>0</v>
       </c>
       <c r="S13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B14" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E14" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G14" t="n">
         <v>3.0</v>
       </c>
       <c r="H14" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I14" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R14" t="b">
         <v>0</v>
       </c>
       <c r="S14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B15" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E15" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G15" t="n">
         <v>3.0</v>
       </c>
       <c r="H15" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="I15" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R15" t="b">
         <v>0</v>
       </c>
       <c r="S15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B16" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E16" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G16" t="n">
         <v>3.0</v>
       </c>
       <c r="H16" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I16" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R16" t="b">
         <v>0</v>
       </c>
       <c r="S16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B17" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D17" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E17" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G17" t="n">
         <v>1.0</v>
       </c>
       <c r="H17" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I17" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R17" t="b">
         <v>0</v>
       </c>
       <c r="S17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B18" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D18" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E18" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G18" t="n">
         <v>2.0</v>
       </c>
       <c r="H18" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="I18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R18" t="b">
         <v>0</v>
       </c>
       <c r="S18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B19" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D19" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E19" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G19" t="n">
         <v>1.0</v>
       </c>
       <c r="H19" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I19" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="Q19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R19" t="b">
         <v>0</v>
       </c>
       <c r="S19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="T19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="V19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -3206,176 +3301,176 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection password="D4D4" sheet="true" scenarios="true" objects="true"/>
   <mergeCells>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -3390,337 +3485,337 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection password="D4D4" sheet="true" scenarios="true" objects="true"/>
   <mergeCells>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -3735,57 +3830,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B3"/>
       <c r="C3" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -3793,16 +3888,17 @@
       <c r="G3"/>
     </row>
   </sheetData>
-  <sheetProtection password="D4D4" sheet="true" scenarios="true" objects="true"/>
   <mergeCells>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
@@ -3817,55 +3913,55 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection password="D4D4" sheet="true" scenarios="true" objects="true"/>
   <mergeCells>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
conf scheduling: Pinned talks only need to be set in the talks sheet. Room view shows solutions
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -11,11 +11,11 @@
     <sheet name="Rooms" r:id="rId5" sheetId="3"/>
     <sheet name="Speakers" r:id="rId6" sheetId="4"/>
     <sheet name="Talks" r:id="rId7" sheetId="5"/>
-    <sheet name="Room view" r:id="rId8" sheetId="6"/>
-    <sheet name="Speaker view" r:id="rId9" sheetId="7"/>
-    <sheet name="Theme view" r:id="rId10" sheetId="8"/>
-    <sheet name="Sector view" r:id="rId11" sheetId="9"/>
-    <sheet name="Content view" r:id="rId12" sheetId="10"/>
+    <sheet name="Rooms view" r:id="rId8" sheetId="6"/>
+    <sheet name="Speakers view" r:id="rId9" sheetId="7"/>
+    <sheet name="Theme tracks view" r:id="rId10" sheetId="8"/>
+    <sheet name="Sectors view" r:id="rId11" sheetId="9"/>
+    <sheet name="Contents view" r:id="rId12" sheetId="10"/>
   </sheets>
 </workbook>
 </file>
@@ -70,10 +70,10 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Theme conflict</t>
-  </si>
-  <si>
-    <t>Soft penalty per common theme of 2 talks that have an overlapping timeslot</t>
+    <t>Theme track conflict</t>
+  </si>
+  <si>
+    <t>Soft penalty per common theme track of 2 talks that have an overlapping timeslot</t>
   </si>
   <si>
     <t>Sector conflict</t>
@@ -214,207 +214,207 @@
     <t>Large, Recorded</t>
   </si>
   <si>
+    <t>R 2</t>
+  </si>
+  <si>
+    <t>R 3</t>
+  </si>
+  <si>
+    <t>Recorded</t>
+  </si>
+  <si>
+    <t>R 4</t>
+  </si>
+  <si>
+    <t>R 5</t>
+  </si>
+  <si>
+    <t>Lab_room, Large, Recorded</t>
+  </si>
+  <si>
+    <t>Required timeslot tags</t>
+  </si>
+  <si>
+    <t>Preferred timeslot tags</t>
+  </si>
+  <si>
+    <t>Prohibited timeslot tags</t>
+  </si>
+  <si>
+    <t>Undesired timeslot tags</t>
+  </si>
+  <si>
+    <t>Required room tags</t>
+  </si>
+  <si>
+    <t>Preferred room tags</t>
+  </si>
+  <si>
+    <t>Prohibited room tags</t>
+  </si>
+  <si>
+    <t>Undesired room tags</t>
+  </si>
+  <si>
+    <t>Amy Cole</t>
+  </si>
+  <si>
+    <t>Beth Fox</t>
+  </si>
+  <si>
+    <t>Chad Green</t>
+  </si>
+  <si>
+    <t>Dan Jones</t>
+  </si>
+  <si>
+    <t>Elsa King</t>
+  </si>
+  <si>
+    <t>Flo Li</t>
+  </si>
+  <si>
+    <t>Gus Poe</t>
+  </si>
+  <si>
+    <t>Hugo Rye</t>
+  </si>
+  <si>
+    <t>Ivy Smith</t>
+  </si>
+  <si>
+    <t>Jay Watt</t>
+  </si>
+  <si>
+    <t>Amy Fox</t>
+  </si>
+  <si>
+    <t>Beth Green</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Speakers</t>
+  </si>
+  <si>
+    <t>Theme track tags</t>
+  </si>
+  <si>
+    <t>Sector tags</t>
+  </si>
+  <si>
+    <t>Audience level</t>
+  </si>
+  <si>
+    <t>Content tags</t>
+  </si>
+  <si>
+    <t>Language</t>
+  </si>
+  <si>
+    <t>Pinned by user</t>
+  </si>
+  <si>
+    <t>Timeslot day</t>
+  </si>
+  <si>
+    <t>Room</t>
+  </si>
+  <si>
+    <t>S00</t>
+  </si>
+  <si>
+    <t>Hands on real-time OpenShift</t>
+  </si>
+  <si>
+    <t>Cloud</t>
+  </si>
+  <si>
+    <t>Government</t>
+  </si>
+  <si>
+    <t>OpenShift, Kubernetes</t>
+  </si>
+  <si>
+    <t>en</t>
+  </si>
+  <si>
+    <t>Lab_room</t>
+  </si>
+  <si>
+    <t>S01</t>
+  </si>
+  <si>
+    <t>Advanced containerized WildFly</t>
+  </si>
+  <si>
+    <t>Big Data</t>
+  </si>
+  <si>
+    <t>WildFly</t>
+  </si>
+  <si>
+    <t>S02</t>
+  </si>
+  <si>
+    <t>Learn virtualized Spring</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>Spring</t>
+  </si>
+  <si>
+    <t>S03</t>
+  </si>
+  <si>
+    <t>Intro to serverless Drools</t>
+  </si>
+  <si>
+    <t>Culture</t>
+  </si>
+  <si>
+    <t>Drools</t>
+  </si>
+  <si>
+    <t>S04</t>
+  </si>
+  <si>
+    <t>Discover AI-driven OptaPlanner</t>
+  </si>
+  <si>
+    <t>Elsa King, Flo Li</t>
+  </si>
+  <si>
+    <t>IoT</t>
+  </si>
+  <si>
+    <t>OptaPlanner</t>
+  </si>
+  <si>
+    <t>S05</t>
+  </si>
+  <si>
+    <t>Mastering machine learning jBPM</t>
+  </si>
+  <si>
+    <t>Gus Poe, Hugo Rye</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>jBPM</t>
+  </si>
+  <si>
     <t>S06</t>
   </si>
   <si>
-    <t>R 2</t>
-  </si>
-  <si>
-    <t>R 3</t>
-  </si>
-  <si>
-    <t>Recorded</t>
-  </si>
-  <si>
-    <t>R 4</t>
-  </si>
-  <si>
-    <t>R 5</t>
-  </si>
-  <si>
-    <t>Lab_room, Large, Recorded</t>
-  </si>
-  <si>
-    <t>Required timeslot tags</t>
-  </si>
-  <si>
-    <t>Preferred timeslot tags</t>
-  </si>
-  <si>
-    <t>Prohibited timeslot tags</t>
-  </si>
-  <si>
-    <t>Undesired timeslot tags</t>
-  </si>
-  <si>
-    <t>Required room tags</t>
-  </si>
-  <si>
-    <t>Preferred room tags</t>
-  </si>
-  <si>
-    <t>Prohibited room tags</t>
-  </si>
-  <si>
-    <t>Undesired room tags</t>
-  </si>
-  <si>
-    <t>Amy Cole</t>
-  </si>
-  <si>
-    <t>Beth Fox</t>
-  </si>
-  <si>
-    <t>Chad Green</t>
-  </si>
-  <si>
-    <t>Dan Jones</t>
-  </si>
-  <si>
-    <t>Elsa King</t>
-  </si>
-  <si>
-    <t>Flo Li</t>
-  </si>
-  <si>
-    <t>Gus Poe</t>
-  </si>
-  <si>
-    <t>Hugo Rye</t>
-  </si>
-  <si>
-    <t>Ivy Smith</t>
-  </si>
-  <si>
-    <t>Jay Watt</t>
-  </si>
-  <si>
-    <t>Amy Fox</t>
-  </si>
-  <si>
-    <t>Beth Green</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>Speakers</t>
-  </si>
-  <si>
-    <t>Theme tags</t>
-  </si>
-  <si>
-    <t>Sector tags</t>
-  </si>
-  <si>
-    <t>Audience level</t>
-  </si>
-  <si>
-    <t>Content tags</t>
-  </si>
-  <si>
-    <t>Language</t>
-  </si>
-  <si>
-    <t>Pinned by user</t>
-  </si>
-  <si>
-    <t>Timeslot day</t>
-  </si>
-  <si>
-    <t>Room</t>
-  </si>
-  <si>
-    <t>S00</t>
-  </si>
-  <si>
-    <t>Hands on real-time OpenShift</t>
-  </si>
-  <si>
-    <t>Cloud</t>
-  </si>
-  <si>
-    <t>Government</t>
-  </si>
-  <si>
-    <t>OpenShift, Kubernetes</t>
-  </si>
-  <si>
-    <t>en</t>
-  </si>
-  <si>
-    <t>Lab_room</t>
-  </si>
-  <si>
-    <t>S01</t>
-  </si>
-  <si>
-    <t>Advanced containerized WildFly</t>
-  </si>
-  <si>
-    <t>Big Data</t>
-  </si>
-  <si>
-    <t>WildFly</t>
-  </si>
-  <si>
-    <t>S02</t>
-  </si>
-  <si>
-    <t>Learn virtualized Spring</t>
-  </si>
-  <si>
-    <t>Mobile</t>
-  </si>
-  <si>
-    <t>Spring</t>
-  </si>
-  <si>
-    <t>S03</t>
-  </si>
-  <si>
-    <t>Intro to serverless Drools</t>
-  </si>
-  <si>
-    <t>Culture</t>
-  </si>
-  <si>
-    <t>Drools</t>
-  </si>
-  <si>
-    <t>S04</t>
-  </si>
-  <si>
-    <t>Discover AI-driven OptaPlanner</t>
-  </si>
-  <si>
-    <t>Elsa King, Flo Li</t>
-  </si>
-  <si>
-    <t>IoT</t>
-  </si>
-  <si>
-    <t>OptaPlanner</t>
-  </si>
-  <si>
-    <t>S05</t>
-  </si>
-  <si>
-    <t>Mastering machine learning jBPM</t>
-  </si>
-  <si>
-    <t>Gus Poe, Hugo Rye</t>
-  </si>
-  <si>
-    <t>Security</t>
-  </si>
-  <si>
-    <t>jBPM</t>
-  </si>
-  <si>
     <t>Tuning IOT-driven Camel</t>
   </si>
   <si>
@@ -550,7 +550,7 @@
     <t>Speaker</t>
   </si>
   <si>
-    <t>Theme tag</t>
+    <t>Theme track tag</t>
   </si>
   <si>
     <t>Sector tag</t>
@@ -1140,8 +1140,8 @@
       <c r="C3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>53</v>
+      <c r="D3" t="s">
+        <v>34</v>
       </c>
       <c r="E3" t="s">
         <v>34</v>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
         <v>34</v>
@@ -1184,10 +1184,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" t="s">
         <v>55</v>
-      </c>
-      <c r="B5" t="s">
-        <v>56</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>34</v>
@@ -1210,10 +1210,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>34</v>
@@ -1236,10 +1236,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" t="s">
         <v>58</v>
-      </c>
-      <c r="B7" t="s">
-        <v>59</v>
       </c>
       <c r="C7" t="s">
         <v>34</v>
@@ -1343,28 +1343,28 @@
         <v>44</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>45</v>
@@ -1387,7 +1387,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
@@ -1434,7 +1434,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B4" t="s">
         <v>34</v>
@@ -1481,7 +1481,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5" t="s">
         <v>34</v>
@@ -1499,7 +1499,7 @@
         <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H5" t="s">
         <v>34</v>
@@ -1528,7 +1528,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
         <v>34</v>
@@ -1575,7 +1575,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
@@ -1622,7 +1622,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B8" t="s">
         <v>34</v>
@@ -1669,7 +1669,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B9" t="s">
         <v>34</v>
@@ -1687,7 +1687,7 @@
         <v>34</v>
       </c>
       <c r="G9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H9" t="s">
         <v>34</v>
@@ -1716,7 +1716,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B10" t="s">
         <v>34</v>
@@ -1763,7 +1763,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B11" t="s">
         <v>34</v>
@@ -1793,7 +1793,7 @@
         <v>34</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>34</v>
@@ -1810,7 +1810,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B12" t="s">
         <v>34</v>
@@ -1828,7 +1828,7 @@
         <v>34</v>
       </c>
       <c r="G12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H12" t="s">
         <v>34</v>
@@ -1857,7 +1857,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B13" t="s">
         <v>34</v>
@@ -1904,7 +1904,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B14" t="s">
         <v>34</v>
@@ -1989,61 +1989,61 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>81</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>26</v>
@@ -2052,51 +2052,51 @@
         <v>27</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" t="s">
         <v>91</v>
-      </c>
-      <c r="B2" t="s">
-        <v>92</v>
       </c>
       <c r="C2" t="s">
         <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" t="s">
         <v>93</v>
-      </c>
-      <c r="F2" t="s">
-        <v>94</v>
       </c>
       <c r="G2" t="n">
         <v>2.0</v>
       </c>
       <c r="H2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I2" t="s">
         <v>95</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" t="s">
+        <v>34</v>
+      </c>
+      <c r="L2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" t="s">
         <v>96</v>
-      </c>
-      <c r="J2" t="s">
-        <v>34</v>
-      </c>
-      <c r="K2" t="s">
-        <v>34</v>
-      </c>
-      <c r="L2" t="s">
-        <v>34</v>
-      </c>
-      <c r="M2" t="s">
-        <v>34</v>
-      </c>
-      <c r="N2" t="s">
-        <v>97</v>
       </c>
       <c r="O2" t="s">
         <v>34</v>
@@ -2125,19 +2125,19 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" t="s">
         <v>98</v>
-      </c>
-      <c r="B3" t="s">
-        <v>99</v>
       </c>
       <c r="C3" t="s">
         <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F3" t="s">
         <v>34</v>
@@ -2146,25 +2146,25 @@
         <v>1.0</v>
       </c>
       <c r="H3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I3" t="s">
+        <v>95</v>
+      </c>
+      <c r="J3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N3" t="s">
         <v>96</v>
-      </c>
-      <c r="J3" t="s">
-        <v>34</v>
-      </c>
-      <c r="K3" t="s">
-        <v>34</v>
-      </c>
-      <c r="L3" t="s">
-        <v>34</v>
-      </c>
-      <c r="M3" t="s">
-        <v>34</v>
-      </c>
-      <c r="N3" t="s">
-        <v>97</v>
       </c>
       <c r="O3" t="s">
         <v>34</v>
@@ -2193,19 +2193,19 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" t="s">
         <v>102</v>
-      </c>
-      <c r="B4" t="s">
-        <v>103</v>
       </c>
       <c r="C4" t="s">
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F4" t="s">
         <v>34</v>
@@ -2214,10 +2214,10 @@
         <v>3.0</v>
       </c>
       <c r="H4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J4" t="s">
         <v>34</v>
@@ -2261,19 +2261,19 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" t="s">
         <v>106</v>
-      </c>
-      <c r="B5" t="s">
-        <v>107</v>
       </c>
       <c r="C5" t="s">
         <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F5" t="s">
         <v>34</v>
@@ -2282,10 +2282,10 @@
         <v>2.0</v>
       </c>
       <c r="H5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J5" t="s">
         <v>34</v>
@@ -2329,19 +2329,19 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" t="s">
         <v>110</v>
-      </c>
-      <c r="B6" t="s">
-        <v>111</v>
       </c>
       <c r="C6" t="s">
         <v>36</v>
       </c>
       <c r="D6" t="s">
+        <v>111</v>
+      </c>
+      <c r="E6" t="s">
         <v>112</v>
-      </c>
-      <c r="E6" t="s">
-        <v>113</v>
       </c>
       <c r="F6" t="s">
         <v>34</v>
@@ -2350,10 +2350,10 @@
         <v>3.0</v>
       </c>
       <c r="H6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J6" t="s">
         <v>34</v>
@@ -2397,19 +2397,19 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B7" t="s">
         <v>115</v>
-      </c>
-      <c r="B7" t="s">
-        <v>116</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
       </c>
       <c r="D7" t="s">
+        <v>116</v>
+      </c>
+      <c r="E7" t="s">
         <v>117</v>
-      </c>
-      <c r="E7" t="s">
-        <v>118</v>
       </c>
       <c r="F7" t="s">
         <v>34</v>
@@ -2418,10 +2418,10 @@
         <v>1.0</v>
       </c>
       <c r="H7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J7" t="s">
         <v>34</v>
@@ -2465,7 +2465,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>119</v>
       </c>
       <c r="B8" t="s">
         <v>120</v>
@@ -2474,7 +2474,7 @@
         <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E8" t="s">
         <v>121</v>
@@ -2489,7 +2489,7 @@
         <v>122</v>
       </c>
       <c r="I8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J8" t="s">
         <v>34</v>
@@ -2542,10 +2542,10 @@
         <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F9" t="s">
         <v>34</v>
@@ -2557,7 +2557,7 @@
         <v>125</v>
       </c>
       <c r="I9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J9" t="s">
         <v>34</v>
@@ -2625,7 +2625,7 @@
         <v>130</v>
       </c>
       <c r="I10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J10" t="s">
         <v>34</v>
@@ -2678,7 +2678,7 @@
         <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E11" t="s">
         <v>121</v>
@@ -2693,7 +2693,7 @@
         <v>133</v>
       </c>
       <c r="I11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J11" t="s">
         <v>34</v>
@@ -2761,7 +2761,7 @@
         <v>138</v>
       </c>
       <c r="I12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J12" t="s">
         <v>34</v>
@@ -2814,10 +2814,10 @@
         <v>36</v>
       </c>
       <c r="D13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E13" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F13" t="s">
         <v>34</v>
@@ -2829,7 +2829,7 @@
         <v>141</v>
       </c>
       <c r="I13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J13" t="s">
         <v>34</v>
@@ -2882,10 +2882,10 @@
         <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F14" t="s">
         <v>34</v>
@@ -2897,7 +2897,7 @@
         <v>144</v>
       </c>
       <c r="I14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J14" t="s">
         <v>34</v>
@@ -2950,10 +2950,10 @@
         <v>36</v>
       </c>
       <c r="D15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" t="s">
         <v>117</v>
-      </c>
-      <c r="E15" t="s">
-        <v>118</v>
       </c>
       <c r="F15" t="s">
         <v>34</v>
@@ -2965,7 +2965,7 @@
         <v>147</v>
       </c>
       <c r="I15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J15" t="s">
         <v>34</v>
@@ -3018,7 +3018,7 @@
         <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E16" t="s">
         <v>150</v>
@@ -3033,7 +3033,7 @@
         <v>151</v>
       </c>
       <c r="I16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J16" t="s">
         <v>34</v>
@@ -3086,10 +3086,10 @@
         <v>36</v>
       </c>
       <c r="D17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F17" t="s">
         <v>34</v>
@@ -3101,7 +3101,7 @@
         <v>154</v>
       </c>
       <c r="I17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J17" t="s">
         <v>34</v>
@@ -3169,7 +3169,7 @@
         <v>158</v>
       </c>
       <c r="I18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J18" t="s">
         <v>34</v>
@@ -3228,7 +3228,7 @@
         <v>162</v>
       </c>
       <c r="F19" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G19" t="n">
         <v>1.0</v>
@@ -3237,7 +3237,7 @@
         <v>163</v>
       </c>
       <c r="I19" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J19" t="s">
         <v>34</v>
@@ -3324,7 +3324,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>45</v>
@@ -3353,7 +3353,7 @@
         <v>34</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>53</v>
+        <v>119</v>
       </c>
       <c r="D3" t="s">
         <v>34</v>
@@ -3370,7 +3370,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>34</v>
@@ -3393,7 +3393,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>34</v>
@@ -3416,7 +3416,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>34</v>
@@ -3439,7 +3439,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
@@ -3531,7 +3531,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
@@ -3554,7 +3554,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B4" t="s">
         <v>34</v>
@@ -3577,7 +3577,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5" t="s">
         <v>34</v>
@@ -3600,7 +3600,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
         <v>34</v>
@@ -3623,7 +3623,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
@@ -3646,7 +3646,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B8" t="s">
         <v>34</v>
@@ -3669,7 +3669,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B9" t="s">
         <v>34</v>
@@ -3692,7 +3692,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B10" t="s">
         <v>34</v>
@@ -3715,13 +3715,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>53</v>
+        <v>119</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>34</v>
@@ -3738,7 +3738,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B12" t="s">
         <v>34</v>
@@ -3761,7 +3761,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B13" t="s">
         <v>34</v>
@@ -3784,7 +3784,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B14" t="s">
         <v>34</v>
@@ -3880,7 +3880,7 @@
       </c>
       <c r="B3"/>
       <c r="C3" s="4" t="s">
-        <v>53</v>
+        <v>119</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>

</xml_diff>

<commit_message>
Add "Audience level diversity" constraint (Mario's request)
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="171">
   <si>
     <t>Conference name</t>
   </si>
@@ -85,7 +85,13 @@
     <t>Content audience level flow violation</t>
   </si>
   <si>
-    <t>Soft penalty per common content of 2 talks with a different audience level for which the easier talk isn't scheduled earlier than the other talk.</t>
+    <t>Soft penalty per common content of 2 talks with a different audience level for which the easier talk isn't scheduled earlier than the other talk</t>
+  </si>
+  <si>
+    <t>Audience level diversity</t>
+  </si>
+  <si>
+    <t>Soft reward per 2 talks that have the same timeslot and a different audience level</t>
   </si>
   <si>
     <t>Language diversity</t>
@@ -682,7 +688,7 @@
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="11.80859375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="130.52734375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="129.94140625" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -743,7 +749,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="n">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>12</v>
@@ -779,12 +785,12 @@
         <v>10.0</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11" t="n">
         <v>10.0</v>
@@ -795,13 +801,13 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B12" t="n">
         <v>10.0</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13">
@@ -823,18 +829,29 @@
         <v>10.0</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B15" t="n">
         <v>10.0</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -859,57 +876,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B3"/>
       <c r="C3" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -940,121 +957,121 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1080,184 +1097,184 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1293,660 +1310,660 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1989,1294 +2006,1294 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="U1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G2" t="n">
         <v>2.0</v>
       </c>
       <c r="H2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="O2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R2" t="b">
         <v>0</v>
       </c>
       <c r="S2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G3" t="n">
         <v>1.0</v>
       </c>
       <c r="H3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="O3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R3" t="b">
         <v>0</v>
       </c>
       <c r="S3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G4" t="n">
         <v>3.0</v>
       </c>
       <c r="H4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R4" t="b">
         <v>0</v>
       </c>
       <c r="S4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G5" t="n">
         <v>2.0</v>
       </c>
       <c r="H5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R5" t="b">
         <v>0</v>
       </c>
       <c r="S5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G6" t="n">
         <v>3.0</v>
       </c>
       <c r="H6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R6" t="b">
         <v>0</v>
       </c>
       <c r="S6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G7" t="n">
         <v>1.0</v>
       </c>
       <c r="H7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R7" t="b">
         <v>0</v>
       </c>
       <c r="S7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G8" t="n">
         <v>1.0</v>
       </c>
       <c r="H8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R8" s="3" t="b">
         <v>1</v>
       </c>
       <c r="S8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="T8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="U8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="V8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E9" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G9" t="n">
         <v>2.0</v>
       </c>
       <c r="H9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R9" t="b">
         <v>0</v>
       </c>
       <c r="S9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G10" t="n">
         <v>3.0</v>
       </c>
       <c r="H10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="I10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R10" t="b">
         <v>0</v>
       </c>
       <c r="S10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E11" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G11" t="n">
         <v>1.0</v>
       </c>
       <c r="H11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R11" t="b">
         <v>0</v>
       </c>
       <c r="S11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E12" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G12" t="n">
         <v>3.0</v>
       </c>
       <c r="H12" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I12" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R12" t="b">
         <v>0</v>
       </c>
       <c r="S12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B13" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D13" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G13" t="n">
         <v>3.0</v>
       </c>
       <c r="H13" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R13" t="b">
         <v>0</v>
       </c>
       <c r="S13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B14" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D14" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E14" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G14" t="n">
         <v>3.0</v>
       </c>
       <c r="H14" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I14" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R14" t="b">
         <v>0</v>
       </c>
       <c r="S14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B15" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D15" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E15" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G15" t="n">
         <v>3.0</v>
       </c>
       <c r="H15" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="I15" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R15" t="b">
         <v>0</v>
       </c>
       <c r="S15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B16" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C16" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E16" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G16" t="n">
         <v>3.0</v>
       </c>
       <c r="H16" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I16" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R16" t="b">
         <v>0</v>
       </c>
       <c r="S16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B17" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C17" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D17" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E17" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G17" t="n">
         <v>1.0</v>
       </c>
       <c r="H17" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="I17" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R17" t="b">
         <v>0</v>
       </c>
       <c r="S17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V17" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B18" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D18" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E18" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G18" t="n">
         <v>2.0</v>
       </c>
       <c r="H18" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R18" t="b">
         <v>0</v>
       </c>
       <c r="S18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B19" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C19" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D19" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E19" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F19" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G19" t="n">
         <v>1.0</v>
       </c>
       <c r="H19" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R19" t="b">
         <v>0</v>
       </c>
       <c r="S19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -3301,163 +3318,163 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -3485,324 +3502,324 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -3830,57 +3847,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B3"/>
       <c r="C3" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -3913,48 +3930,48 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
conf scheduling: define all hard constraint names and explain in xlsx
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -32,7 +32,7 @@
   Ivy Smith
   PINNED BY USER
 Constraint matches:
-  Speaker unavailable timeslots (S06): -1hard</t>
+  Speaker unavailable timeslot (S06): -1hard</t>
       </text>
     </comment>
   </commentList>
@@ -51,7 +51,7 @@
   Ivy Smith
   PINNED BY USER
 Constraint matches:
-  Speaker unavailable timeslots (S06): -1hard</t>
+  Speaker unavailable timeslot (S06): -1hard</t>
       </text>
     </comment>
   </commentList>
@@ -70,7 +70,7 @@
   Ivy Smith
   PINNED BY USER
 Constraint matches:
-  Speaker unavailable timeslots (S06): -1hard</t>
+  Speaker unavailable timeslot (S06): -1hard</t>
       </text>
     </comment>
   </commentList>
@@ -89,7 +89,7 @@
   Ivy Smith
   PINNED BY USER
 Constraint matches:
-  Speaker unavailable timeslots (S06): -1hard</t>
+  Speaker unavailable timeslot (S06): -1hard</t>
       </text>
     </comment>
   </commentList>
@@ -97,7 +97,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="917" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="195">
   <si>
     <t>Conference name</t>
   </si>
@@ -178,6 +178,75 @@
   </si>
   <si>
     <t>Talk undesired room tag</t>
+  </si>
+  <si>
+    <t>Talk type of timeslot</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>Hard penalty per talk in a timeslot with an other talk type</t>
+  </si>
+  <si>
+    <t>Room unavailable timeslot</t>
+  </si>
+  <si>
+    <t>Hard penalty per talk with an unavailable room at its timeslot</t>
+  </si>
+  <si>
+    <t>Room conflict</t>
+  </si>
+  <si>
+    <t>Hard penalty per pair of talks in the same room in overlapping timeslots</t>
+  </si>
+  <si>
+    <t>Speaker unavailable timeslot</t>
+  </si>
+  <si>
+    <t>Hard penalty per talk with an unavailable speaker at its timeslot</t>
+  </si>
+  <si>
+    <t>Speaker conflict</t>
+  </si>
+  <si>
+    <t>Hard penalty per pair of talks with the same speaker in overlapping timeslots</t>
+  </si>
+  <si>
+    <t>Speaker required timeslot tag</t>
+  </si>
+  <si>
+    <t>Hard penalty per missing required tag in a talk's timeslot</t>
+  </si>
+  <si>
+    <t>Speaker prohibited timeslot tag</t>
+  </si>
+  <si>
+    <t>Hard penalty per prohibited tag in a talk's timeslot</t>
+  </si>
+  <si>
+    <t>Talk required timeslot tag</t>
+  </si>
+  <si>
+    <t>Talk prohibited timeslot tag</t>
+  </si>
+  <si>
+    <t>Speaker required room tag</t>
+  </si>
+  <si>
+    <t>Hard penalty per missing required tag in a talk's room</t>
+  </si>
+  <si>
+    <t>Speaker prohibited room tag</t>
+  </si>
+  <si>
+    <t>Hard penalty per prohibited tag in a talk's room</t>
+  </si>
+  <si>
+    <t>Talk required room tag</t>
+  </si>
+  <si>
+    <t>Talk prohibited room tag</t>
   </si>
   <si>
     <t>Day</t>
@@ -917,6 +986,150 @@
         <v>24</v>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <drawing r:id="rId1"/>
@@ -942,71 +1155,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>171</v>
+        <v>194</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1033,121 +1246,121 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>31</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>42</v>
+        <v>65</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1173,184 +1386,184 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1386,660 +1599,660 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -2082,1294 +2295,1294 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="O1" s="1" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R2" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R3" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R4" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>107</v>
+        <v>130</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R5" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V5" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R6" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>118</v>
+        <v>141</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="H7" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="I7" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="J7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R7" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V7" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R8" s="4" t="b">
         <v>1</v>
       </c>
       <c r="S8" s="2" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="U8" s="2" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="V8" s="2" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R9" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V9" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>128</v>
+        <v>151</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>129</v>
+        <v>152</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R10" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V10" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>134</v>
+        <v>157</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R11" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V11" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>139</v>
+        <v>162</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R12" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V12" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>142</v>
+        <v>165</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>143</v>
+        <v>166</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R13" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V13" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>144</v>
+        <v>167</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>145</v>
+        <v>168</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R14" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>147</v>
+        <v>170</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>148</v>
+        <v>171</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>118</v>
+        <v>141</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>149</v>
+        <v>172</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R15" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V15" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>150</v>
+        <v>173</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>151</v>
+        <v>174</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R16" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V16" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R17" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V17" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>157</v>
+        <v>180</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>160</v>
+        <v>183</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R18" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V18" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>162</v>
+        <v>185</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="R19" s="2" t="b">
         <v>0</v>
       </c>
       <c r="S19" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="T19" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="U19" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="V19" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -3404,163 +3617,163 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" ht="30.0" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" ht="30.0" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" ht="30.0" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" ht="30.0" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" ht="30.0" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -3592,324 +3805,324 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" ht="15.0" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="true">
       <c r="A8" s="2" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="true">
       <c r="A9" s="2" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" ht="15.0" customHeight="true">
       <c r="A10" s="2" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" ht="15.0" customHeight="true">
       <c r="A11" s="2" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="true">
       <c r="A12" s="2" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" ht="15.0" customHeight="true">
       <c r="A13" s="2" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" ht="15.0" customHeight="true">
       <c r="A14" s="2" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -3941,71 +4154,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>168</v>
+        <v>191</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -4037,48 +4250,48 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>169</v>
+        <v>192</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
conf scheduling: introduce talk type set (for RH Summit)
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -125,7 +125,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="210">
   <si>
     <t>Conference name</t>
   </si>
@@ -304,163 +304,166 @@
     <t>End</t>
   </si>
   <si>
+    <t>Talk types</t>
+  </si>
+  <si>
+    <t>Tags</t>
+  </si>
+  <si>
+    <t>Mon 2018-10-01</t>
+  </si>
+  <si>
+    <t>10:15</t>
+  </si>
+  <si>
+    <t>12:15</t>
+  </si>
+  <si>
+    <t>Lab</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>11:00</t>
+  </si>
+  <si>
+    <t>Breakout</t>
+  </si>
+  <si>
+    <t>11:30</t>
+  </si>
+  <si>
+    <t>13:00</t>
+  </si>
+  <si>
+    <t>15:00</t>
+  </si>
+  <si>
+    <t>15:30</t>
+  </si>
+  <si>
+    <t>16:15</t>
+  </si>
+  <si>
+    <t>16:30</t>
+  </si>
+  <si>
+    <t>17:15</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>10:15-12:15</t>
+  </si>
+  <si>
+    <t>10:15-11:00</t>
+  </si>
+  <si>
+    <t>11:30-12:15</t>
+  </si>
+  <si>
+    <t>13:00-15:00</t>
+  </si>
+  <si>
+    <t>15:30-16:15</t>
+  </si>
+  <si>
+    <t>16:30-17:15</t>
+  </si>
+  <si>
+    <t>R 1</t>
+  </si>
+  <si>
+    <t>Large, Recorded</t>
+  </si>
+  <si>
+    <t>R 2</t>
+  </si>
+  <si>
+    <t>R 3</t>
+  </si>
+  <si>
+    <t>Recorded</t>
+  </si>
+  <si>
+    <t>R 4</t>
+  </si>
+  <si>
+    <t>R 5</t>
+  </si>
+  <si>
+    <t>Lab_room, Large, Recorded</t>
+  </si>
+  <si>
+    <t>Required timeslot tags</t>
+  </si>
+  <si>
+    <t>Preferred timeslot tags</t>
+  </si>
+  <si>
+    <t>Prohibited timeslot tags</t>
+  </si>
+  <si>
+    <t>Undesired timeslot tags</t>
+  </si>
+  <si>
+    <t>Required room tags</t>
+  </si>
+  <si>
+    <t>Preferred room tags</t>
+  </si>
+  <si>
+    <t>Prohibited room tags</t>
+  </si>
+  <si>
+    <t>Undesired room tags</t>
+  </si>
+  <si>
+    <t>Amy Cole</t>
+  </si>
+  <si>
+    <t>Beth Fox</t>
+  </si>
+  <si>
+    <t>Chad Green</t>
+  </si>
+  <si>
+    <t>Dan Jones</t>
+  </si>
+  <si>
+    <t>Elsa King</t>
+  </si>
+  <si>
+    <t>Flo Li</t>
+  </si>
+  <si>
+    <t>Gus Poe</t>
+  </si>
+  <si>
+    <t>Hugo Rye</t>
+  </si>
+  <si>
+    <t>Ivy Smith</t>
+  </si>
+  <si>
+    <t>Jay Watt</t>
+  </si>
+  <si>
+    <t>Amy Fox</t>
+  </si>
+  <si>
+    <t>Beth Green</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
     <t>Talk type</t>
-  </si>
-  <si>
-    <t>Tags</t>
-  </si>
-  <si>
-    <t>Mon 2018-10-01</t>
-  </si>
-  <si>
-    <t>10:15</t>
-  </si>
-  <si>
-    <t>12:15</t>
-  </si>
-  <si>
-    <t>Lab</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>11:00</t>
-  </si>
-  <si>
-    <t>Breakout</t>
-  </si>
-  <si>
-    <t>11:30</t>
-  </si>
-  <si>
-    <t>13:00</t>
-  </si>
-  <si>
-    <t>15:00</t>
-  </si>
-  <si>
-    <t>15:30</t>
-  </si>
-  <si>
-    <t>16:15</t>
-  </si>
-  <si>
-    <t>16:30</t>
-  </si>
-  <si>
-    <t>17:15</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>10:15-12:15</t>
-  </si>
-  <si>
-    <t>10:15-11:00</t>
-  </si>
-  <si>
-    <t>11:30-12:15</t>
-  </si>
-  <si>
-    <t>13:00-15:00</t>
-  </si>
-  <si>
-    <t>15:30-16:15</t>
-  </si>
-  <si>
-    <t>16:30-17:15</t>
-  </si>
-  <si>
-    <t>R 1</t>
-  </si>
-  <si>
-    <t>Large, Recorded</t>
-  </si>
-  <si>
-    <t>R 2</t>
-  </si>
-  <si>
-    <t>R 3</t>
-  </si>
-  <si>
-    <t>Recorded</t>
-  </si>
-  <si>
-    <t>R 4</t>
-  </si>
-  <si>
-    <t>R 5</t>
-  </si>
-  <si>
-    <t>Lab_room, Large, Recorded</t>
-  </si>
-  <si>
-    <t>Required timeslot tags</t>
-  </si>
-  <si>
-    <t>Preferred timeslot tags</t>
-  </si>
-  <si>
-    <t>Prohibited timeslot tags</t>
-  </si>
-  <si>
-    <t>Undesired timeslot tags</t>
-  </si>
-  <si>
-    <t>Required room tags</t>
-  </si>
-  <si>
-    <t>Preferred room tags</t>
-  </si>
-  <si>
-    <t>Prohibited room tags</t>
-  </si>
-  <si>
-    <t>Undesired room tags</t>
-  </si>
-  <si>
-    <t>Amy Cole</t>
-  </si>
-  <si>
-    <t>Beth Fox</t>
-  </si>
-  <si>
-    <t>Chad Green</t>
-  </si>
-  <si>
-    <t>Dan Jones</t>
-  </si>
-  <si>
-    <t>Elsa King</t>
-  </si>
-  <si>
-    <t>Flo Li</t>
-  </si>
-  <si>
-    <t>Gus Poe</t>
-  </si>
-  <si>
-    <t>Hugo Rye</t>
-  </si>
-  <si>
-    <t>Ivy Smith</t>
-  </si>
-  <si>
-    <t>Jay Watt</t>
-  </si>
-  <si>
-    <t>Amy Fox</t>
-  </si>
-  <si>
-    <t>Beth Green</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>Title</t>
   </si>
   <si>
     <t>Speakers</t>
@@ -1290,7 +1293,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>
@@ -1313,13 +1316,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -1386,7 +1389,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>
@@ -1409,13 +1412,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -1482,7 +1485,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>
@@ -1505,13 +1508,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -1544,7 +1547,7 @@
     <col min="1" max="1" width="15.99609375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="6.0859375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="6.0859375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="9.41796875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="10.29296875" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="5.1484375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
@@ -2606,28 +2609,28 @@
         <v>111</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>112</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>90</v>
@@ -2654,10 +2657,10 @@
         <v>97</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>57</v>
@@ -2666,15 +2669,15 @@
         <v>58</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>64</v>
@@ -2683,22 +2686,22 @@
         <v>98</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>65</v>
@@ -2713,7 +2716,7 @@
         <v>65</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>65</v>
@@ -2742,10 +2745,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>64</v>
@@ -2754,22 +2757,22 @@
         <v>99</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>65</v>
@@ -2784,7 +2787,7 @@
         <v>65</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>65</v>
@@ -2813,10 +2816,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>67</v>
@@ -2825,22 +2828,22 @@
         <v>100</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>65</v>
@@ -2884,10 +2887,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>67</v>
@@ -2896,22 +2899,22 @@
         <v>101</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>65</v>
@@ -2955,34 +2958,34 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>65</v>
@@ -3026,34 +3029,34 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>65</v>
@@ -3097,10 +3100,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>67</v>
@@ -3109,22 +3112,22 @@
         <v>106</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>65</v>
@@ -3168,34 +3171,34 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>65</v>
@@ -3239,34 +3242,34 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>65</v>
@@ -3310,10 +3313,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>67</v>
@@ -3322,22 +3325,22 @@
         <v>102</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>65</v>
@@ -3381,10 +3384,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>67</v>
@@ -3393,22 +3396,22 @@
         <v>103</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>65</v>
@@ -3452,34 +3455,34 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>65</v>
@@ -3523,10 +3526,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>67</v>
@@ -3535,22 +3538,22 @@
         <v>106</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>65</v>
@@ -3594,34 +3597,34 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>65</v>
@@ -3665,34 +3668,34 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>65</v>
@@ -3736,34 +3739,34 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>65</v>
@@ -3807,10 +3810,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>67</v>
@@ -3819,22 +3822,22 @@
         <v>101</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>65</v>
@@ -3878,34 +3881,34 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K19" s="2" t="s">
         <v>65</v>
@@ -4002,7 +4005,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>
@@ -4031,7 +4034,7 @@
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -4190,7 +4193,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>
@@ -4288,7 +4291,7 @@
         <v>65</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>65</v>
@@ -4539,7 +4542,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>
@@ -4562,13 +4565,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -4635,7 +4638,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>

</xml_diff>

<commit_message>
conf scheduling: talkTypeSet on timeslot and room
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -11,32 +11,16 @@
     <sheet name="Rooms" r:id="rId5" sheetId="3"/>
     <sheet name="Speakers" r:id="rId6" sheetId="4"/>
     <sheet name="Talks" r:id="rId7" sheetId="5"/>
-    <sheet name="Rooms view" r:id="rId8" sheetId="6"/>
-    <sheet name="Speakers view" r:id="rId9" sheetId="7"/>
-    <sheet name="Theme tracks view" r:id="rId10" sheetId="8"/>
-    <sheet name="Sectors view" r:id="rId11" sheetId="9"/>
-    <sheet name="Audience type view" r:id="rId12" sheetId="10"/>
-    <sheet name="Audience level view" r:id="rId13" sheetId="11"/>
-    <sheet name="Contents view" r:id="rId14" sheetId="12"/>
+    <sheet name="Score view" r:id="rId8" sheetId="6"/>
+    <sheet name="Rooms view" r:id="rId9" sheetId="7"/>
+    <sheet name="Speakers view" r:id="rId10" sheetId="8"/>
+    <sheet name="Theme tracks view" r:id="rId11" sheetId="9"/>
+    <sheet name="Sectors view" r:id="rId12" sheetId="10"/>
+    <sheet name="Audience type view" r:id="rId13" sheetId="11"/>
+    <sheet name="Audience level view" r:id="rId14" sheetId="12"/>
+    <sheet name="Contents view" r:id="rId15" sheetId="13"/>
   </sheets>
 </workbook>
-</file>
-
-<file path=xl/comments10.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author/>
-  </authors>
-  <commentList>
-    <comment ref="C3" authorId="0">
-      <text>
-        <t>S03: Intro to serverless Drools
-  Dan Jones
-  PINNED BY USER</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/comments11.xml><?xml version="1.0" encoding="utf-8"?>
@@ -73,7 +57,7 @@
 </comments>
 </file>
 
-<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments13.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
@@ -96,6 +80,23 @@
     <author/>
   </authors>
   <commentList>
+    <comment ref="C3" authorId="0">
+      <text>
+        <t>S03: Intro to serverless Drools
+  Dan Jones
+  PINNED BY USER</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
     <comment ref="C6" authorId="0">
       <text>
         <t>S03: Intro to serverless Drools
@@ -107,7 +108,7 @@
 </comments>
 </file>
 
-<file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments9.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
@@ -125,7 +126,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="214">
   <si>
     <t>Conference name</t>
   </si>
@@ -394,9 +395,6 @@
     <t>R 5</t>
   </si>
   <si>
-    <t>Lab_room, Large, Recorded</t>
-  </si>
-  <si>
     <t>Required timeslot tags</t>
   </si>
   <si>
@@ -517,9 +515,6 @@
     <t>en</t>
   </si>
   <si>
-    <t>Lab_room</t>
-  </si>
-  <si>
     <t>S01</t>
   </si>
   <si>
@@ -731,6 +726,24 @@
   </si>
   <si>
     <t>VertX</t>
+  </si>
+  <si>
+    <t>Score</t>
+  </si>
+  <si>
+    <t>-34init</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Usable timeslots</t>
+  </si>
+  <si>
+    <t>Usable rooms</t>
+  </si>
+  <si>
+    <t>Usable sessions</t>
   </si>
   <si>
     <t>S03: Intro to serverless Drools
@@ -863,6 +876,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
 </file>
 
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing"/>
 </file>
@@ -1259,6 +1276,78 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
+    <col min="1" max="1" width="10.23828125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FCE94F"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
     <col min="1" max="1" width="14.1953125" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
@@ -1293,7 +1382,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>
@@ -1316,13 +1405,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -1347,7 +1436,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FCE94F"/>
@@ -1389,7 +1478,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>
@@ -1412,13 +1501,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -1443,7 +1532,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FCE94F"/>
@@ -1485,7 +1574,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>
@@ -1508,13 +1597,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -1682,13 +1771,14 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="6.48828125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="25.6328125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="10.29296875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="15.51171875" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="11.86328125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="11.86328125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1699,11 +1789,11 @@
         <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="E1" s="1" t="s">
         <v>65</v>
       </c>
@@ -1714,6 +1804,9 @@
         <v>65</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1722,24 +1815,27 @@
         <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1748,24 +1844,27 @@
         <v>82</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>65</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G3" s="2" t="s">
+      <c r="F3" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>65</v>
       </c>
       <c r="H3" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1774,24 +1873,27 @@
         <v>84</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D4" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>65</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G4" s="2" t="s">
+      <c r="F4" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>65</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1800,24 +1902,27 @@
         <v>85</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>65</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G5" s="2" t="s">
+      <c r="F5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>65</v>
       </c>
       <c r="H5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1826,24 +1931,27 @@
         <v>87</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>65</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G6" s="2" t="s">
+      <c r="F6" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>65</v>
       </c>
       <c r="H6" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1852,30 +1960,33 @@
         <v>88</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D7" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>65</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="G7" s="3" t="s">
+      <c r="F7" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>65</v>
       </c>
       <c r="H7" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="I7" s="3" t="s">
         <v>65</v>
       </c>
     </row>
   </sheetData>
   <mergeCells>
-    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="D1:I1"/>
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <drawing r:id="rId1"/>
@@ -1956,28 +2067,28 @@
         <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>76</v>
@@ -2000,7 +2111,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>65</v>
@@ -2047,7 +2158,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>65</v>
@@ -2094,7 +2205,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>65</v>
@@ -2141,7 +2252,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>65</v>
@@ -2188,7 +2299,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>65</v>
@@ -2235,7 +2346,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>65</v>
@@ -2282,7 +2393,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>65</v>
@@ -2329,7 +2440,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>65</v>
@@ -2376,7 +2487,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>65</v>
@@ -2423,7 +2534,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>65</v>
@@ -2470,7 +2581,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>65</v>
@@ -2517,7 +2628,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>65</v>
@@ -2603,64 +2714,64 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>121</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>57</v>
@@ -2669,40 +2780,40 @@
         <v>58</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>64</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I2" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="J2" s="2" t="s">
-        <v>129</v>
-      </c>
       <c r="K2" s="2" t="s">
         <v>65</v>
       </c>
@@ -2716,7 +2827,7 @@
         <v>65</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>65</v>
@@ -2745,34 +2856,34 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>64</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>65</v>
@@ -2787,7 +2898,7 @@
         <v>65</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>65</v>
@@ -2816,34 +2927,34 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>65</v>
@@ -2887,34 +2998,34 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>65</v>
@@ -2958,34 +3069,34 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>65</v>
@@ -3029,34 +3140,34 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>65</v>
@@ -3100,34 +3211,34 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>65</v>
@@ -3171,34 +3282,34 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>65</v>
@@ -3242,34 +3353,34 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>65</v>
@@ -3313,34 +3424,34 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>65</v>
@@ -3384,34 +3495,34 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>65</v>
@@ -3455,34 +3566,34 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>65</v>
@@ -3526,34 +3637,34 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>65</v>
@@ -3597,34 +3708,34 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>65</v>
@@ -3668,34 +3779,34 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>65</v>
@@ -3739,34 +3850,34 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>65</v>
@@ -3810,34 +3921,34 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>65</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>65</v>
@@ -3881,34 +3992,34 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E19" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>126</v>
-      </c>
       <c r="G19" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K19" s="2" t="s">
         <v>65</v>
@@ -3957,6 +4068,87 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FCE94F"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="9.4453125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="6.83984375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="16.22265625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="13.59375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="15.30078125" customWidth="true" bestFit="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>16.0</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>16.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FCE94F"/>
@@ -4005,7 +4197,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>
@@ -4034,7 +4226,7 @@
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -4151,7 +4343,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FCE94F"/>
@@ -4193,7 +4385,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>
@@ -4216,7 +4408,7 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>65</v>
@@ -4239,7 +4431,7 @@
     </row>
     <row r="4" ht="15.0" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>65</v>
@@ -4262,7 +4454,7 @@
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>65</v>
@@ -4285,13 +4477,13 @@
     </row>
     <row r="6" ht="15.0" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>65</v>
@@ -4308,7 +4500,7 @@
     </row>
     <row r="7" ht="15.0" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>65</v>
@@ -4331,7 +4523,7 @@
     </row>
     <row r="8" ht="15.0" customHeight="true">
       <c r="A8" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>65</v>
@@ -4354,7 +4546,7 @@
     </row>
     <row r="9" ht="15.0" customHeight="true">
       <c r="A9" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>65</v>
@@ -4377,7 +4569,7 @@
     </row>
     <row r="10" ht="15.0" customHeight="true">
       <c r="A10" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>65</v>
@@ -4400,7 +4592,7 @@
     </row>
     <row r="11" ht="15.0" customHeight="true">
       <c r="A11" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>65</v>
@@ -4423,7 +4615,7 @@
     </row>
     <row r="12" ht="15.0" customHeight="true">
       <c r="A12" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>65</v>
@@ -4446,7 +4638,7 @@
     </row>
     <row r="13" ht="15.0" customHeight="true">
       <c r="A13" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>65</v>
@@ -4469,7 +4661,7 @@
     </row>
     <row r="14" ht="15.0" customHeight="true">
       <c r="A14" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>65</v>
@@ -4500,7 +4692,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FCE94F"/>
@@ -4542,7 +4734,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>76</v>
@@ -4565,13 +4757,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>65</v>
@@ -4594,76 +4786,4 @@
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr>
-    <tabColor rgb="FCE94F"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0"/>
-  <cols>
-    <col min="1" max="1" width="10.23828125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="11.86328125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="11.86328125" customWidth="true" bestFit="true"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells>
-    <mergeCell ref="B1:G1"/>
-  </mergeCells>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Parametrize hard constraints in ConferenceScheduling example
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -152,7 +152,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1066" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="220">
   <si>
     <t>Conference name</t>
   </si>
@@ -256,10 +256,13 @@
     <t>Talk type of timeslot</t>
   </si>
   <si>
-    <t>n/a</t>
-  </si>
-  <si>
-    <t>Hard penalty per talk in a timeslot with an other talk type</t>
+    <t>Hard penalty per talk in a timeslot with another talk type</t>
+  </si>
+  <si>
+    <t>Talk type of room</t>
+  </si>
+  <si>
+    <t>Hard penalty per talk in a room with another talk type</t>
   </si>
   <si>
     <t>Room unavailable timeslot</t>
@@ -1180,143 +1183,154 @@
       <c r="A21" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="2" t="n">
+        <v>10000.0</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>10000.0</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>10000.0</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>34</v>
+      <c r="B29" s="2" t="n">
+        <v>1.0</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>34</v>
+      <c r="B30" s="2" t="n">
+        <v>1.0</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>34</v>
+      <c r="B33" s="2" t="n">
+        <v>1.0</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1344,48 +1358,48 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1416,71 +1430,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1512,71 +1526,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1608,71 +1622,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1704,77 +1718,77 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -1803,13 +1817,13 @@
     <row r="1"/>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -1832,121 +1846,121 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="E4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1973,205 +1987,205 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2207,660 +2221,660 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2904,1351 +2918,1351 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S2" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S3" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W3" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S4" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S5" s="4" t="b">
         <v>1</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="U5" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="V5" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="W5" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S6" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S7" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W7" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S8" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W8" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S9" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W9" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S10" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W10" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S11" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S12" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W12" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S13" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S14" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W14" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S15" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S16" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S17" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W17" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S18" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S19" s="2" t="b">
         <v>0</v>
       </c>
       <c r="T19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="W19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -4274,33 +4288,33 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>2.0</v>
@@ -4317,7 +4331,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>16.0</v>
@@ -4335,7 +4349,7 @@
     <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>18.0</v>
@@ -4382,163 +4396,163 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" ht="45.0" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" ht="45.0" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" ht="45.0" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" ht="45.0" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" ht="45.0" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -4577,324 +4591,324 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" ht="15.0" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="true">
       <c r="A8" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="true">
       <c r="A9" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" ht="15.0" customHeight="true">
       <c r="A10" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" ht="15.0" customHeight="true">
       <c r="A11" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="true">
       <c r="A12" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" ht="15.0" customHeight="true">
       <c r="A13" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" ht="15.0" customHeight="true">
       <c r="A14" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -4926,71 +4940,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Genereate new examples data with the new constraints
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -152,7 +152,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="228">
   <si>
     <t>Conference name</t>
   </si>
@@ -253,6 +253,12 @@
     <t>Talk undesired room tag</t>
   </si>
   <si>
+    <t>Same day talks</t>
+  </si>
+  <si>
+    <t>Soft penalty per common content/theme of 2 talks that are scheduled on different days</t>
+  </si>
+  <si>
     <t>Talk type of timeslot</t>
   </si>
   <si>
@@ -325,6 +331,18 @@
     <t>Talk prohibited room tag</t>
   </si>
   <si>
+    <t>Talk mutually-exclusive-talks tag</t>
+  </si>
+  <si>
+    <t>Hard penalty per two talks that share the same Mutually exclusive talks tag that are scheduled in overlapping timeslots</t>
+  </si>
+  <si>
+    <t>Talk prerequisite talks</t>
+  </si>
+  <si>
+    <t>Hard penalty per talk that is scheduled before any of its prerequisite talks</t>
+  </si>
+  <si>
     <t>Day</t>
   </si>
   <si>
@@ -512,6 +530,12 @@
   </si>
   <si>
     <t>Language</t>
+  </si>
+  <si>
+    <t>Mutually exclusive talks tags</t>
+  </si>
+  <si>
+    <t>Prerequisite talks codes</t>
   </si>
   <si>
     <t>Pinned by user</t>
@@ -1178,18 +1202,18 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" s="1" t="s">
+    <row r="20">
+      <c r="A20" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="2" t="n">
-        <v>10000.0</v>
-      </c>
-      <c r="C21" s="1" t="s">
+      <c r="B20" s="2" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>34</v>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="1" t="s">
         <v>35</v>
@@ -1217,7 +1241,7 @@
         <v>39</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>10.0</v>
+        <v>10000.0</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>40</v>
@@ -1228,7 +1252,7 @@
         <v>41</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1.0</v>
+        <v>10.0</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>42</v>
@@ -1275,12 +1299,12 @@
         <v>1.0</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>1.0</v>
@@ -1291,13 +1315,13 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32">
@@ -1319,18 +1343,51 @@
         <v>1.0</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>54</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1358,48 +1415,48 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1430,71 +1487,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1526,71 +1583,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1622,71 +1679,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1718,77 +1775,77 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -1817,13 +1874,13 @@
     <row r="1"/>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -1846,121 +1903,121 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>68</v>
-      </c>
       <c r="E7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1987,205 +2044,205 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -2221,660 +2278,660 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -2909,1360 +2966,1476 @@
     <col min="16" max="16" width="22.20703125" customWidth="true" bestFit="true"/>
     <col min="17" max="17" width="23.125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="22.84375" customWidth="true" bestFit="true"/>
-    <col min="19" max="19" width="16.65234375" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="16.14453125" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="6.3984375" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" width="6.32421875" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" width="7.02734375" customWidth="true" bestFit="true"/>
+    <col min="19" max="19" width="31.2734375" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="26.23046875" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="16.65234375" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="16.14453125" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" width="6.3984375" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="6.32421875" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="7.02734375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>58</v>
+        <v>128</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>59</v>
+        <v>129</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>122</v>
+        <v>64</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S2" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U2" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T2" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V2" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S3" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U3" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T3" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W3" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S4" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U4" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T4" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U4" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>134</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S5" s="4" t="b">
+        <v>72</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U5" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T5" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="U5" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="V5" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="W5" s="2" t="s">
-        <v>83</v>
+        <v>69</v>
+      </c>
+      <c r="X5" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S6" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U6" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T6" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U6" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S7" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U7" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T7" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U7" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W7" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S8" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U8" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T8" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U8" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W8" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y8" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S9" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U9" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T9" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U9" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W9" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X9" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y9" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S10" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S10" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U10" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T10" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U10" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W10" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X10" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y10" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S11" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S11" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U11" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T11" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U11" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W11" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X11" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y11" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S12" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U12" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T12" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U12" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W12" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y12" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S13" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U13" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T13" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U13" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W13" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y13" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S14" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S14" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U14" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T14" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U14" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W14" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X14" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y14" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S15" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U15" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T15" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U15" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V15" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W15" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X15" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y15" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R16" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S16" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S16" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U16" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T16" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U16" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V16" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W16" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X16" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y16" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R17" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S17" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S17" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T17" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U17" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T17" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U17" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V17" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W17" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X17" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y17" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R18" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S18" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U18" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T18" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U18" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V18" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W18" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y18" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="R19" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="S19" s="2" t="b">
+        <v>72</v>
+      </c>
+      <c r="S19" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T19" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U19" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="T19" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U19" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="V19" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="W19" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
+      </c>
+      <c r="X19" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="Y19" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -4288,33 +4461,33 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>2.0</v>
@@ -4331,7 +4504,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>16.0</v>
@@ -4349,7 +4522,7 @@
     <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>18.0</v>
@@ -4396,163 +4569,163 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" ht="45.0" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" ht="45.0" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" ht="45.0" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" ht="45.0" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" ht="45.0" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -4591,324 +4764,324 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" ht="15.0" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="true">
       <c r="A8" s="2" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="true">
       <c r="A9" s="2" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" ht="15.0" customHeight="true">
       <c r="A10" s="2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" ht="15.0" customHeight="true">
       <c r="A11" s="2" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="true">
       <c r="A12" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" ht="15.0" customHeight="true">
       <c r="A13" s="2" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" ht="15.0" customHeight="true">
       <c r="A14" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -4940,71 +5113,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add capacity field to class Room
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" state="visible" r:id="rId2"/>
@@ -47,7 +47,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">S11: Understand mobile Errai
+          <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
 </t>
@@ -72,7 +72,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">S11: Understand mobile Errai
+          <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
 </t>
@@ -97,7 +97,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">S11: Understand mobile Errai
+          <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
 </t>
@@ -122,7 +122,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">S11: Understand mobile Errai
+          <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
 </t>
@@ -147,7 +147,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">S11: Understand mobile Errai
+          <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
 </t>
@@ -172,7 +172,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">S11: Understand mobile Errai
+          <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
 </t>
@@ -197,7 +197,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">S11: Understand mobile Errai
+          <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
 </t>
@@ -209,7 +209,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="231">
   <si>
     <t xml:space="preserve">Conference name</t>
   </si>
@@ -457,6 +457,9 @@
     <t xml:space="preserve">Name</t>
   </si>
   <si>
+    <t xml:space="preserve">Capacity</t>
+  </si>
+  <si>
     <t xml:space="preserve">10:15-12:15</t>
   </si>
   <si>
@@ -487,12 +490,12 @@
     <t xml:space="preserve">R 3</t>
   </si>
   <si>
+    <t xml:space="preserve">R 4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Recorded</t>
   </si>
   <si>
-    <t xml:space="preserve">R 4</t>
-  </si>
-  <si>
     <t xml:space="preserve">R 5</t>
   </si>
   <si>
@@ -613,231 +616,234 @@
     <t xml:space="preserve">Hands on real-time OpenShift</t>
   </si>
   <si>
+    <t xml:space="preserve">Amy Cole, Beth Fox</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Big Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Business analysts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenShift</t>
+  </si>
+  <si>
+    <t xml:space="preserve">en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advanced containerized WildFly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chad Green, Dan Jones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transportation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Managers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WildFly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Learn virtualized Spring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IoT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programmers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intro to serverless Drools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Big Data, Culture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discover AI-driven OptaPlanner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gus Poe, Hugo Rye</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OptaPlanner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mastering machine learning jBPM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Middleware, Modern Web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financial services</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jBPM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tuning IOT-driven Camel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Government</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Building deep learning XStream</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amy Fox, Beth Green, Amy Cole</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cloud</t>
   </si>
   <si>
-    <t xml:space="preserve">Government</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Business analysts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OpenShift</t>
-  </si>
-  <si>
-    <t xml:space="preserve">en</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Advanced containerized WildFly</t>
+    <t xml:space="preserve">XStream</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Securing scalable Docker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Security, Culture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Docker, Kubernetes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debug enterprise Hibernate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Culture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Telecommunications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hibernate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prepare for streaming GWT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GWT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Understand mobile Errai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elsa King, Flo Li</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Artificial Intelligence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Errai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applying modern Angular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grok distributed Weld</t>
   </si>
   <si>
     <t xml:space="preserve">Middleware, Security</t>
   </si>
   <si>
-    <t xml:space="preserve">Managers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WildFly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Learn virtualized Spring</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chad Green, Dan Jones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Big Data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spring</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Intro to serverless Drools</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drools</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Discover AI-driven OptaPlanner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Artificial Intelligence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OptaPlanner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mastering machine learning jBPM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IoT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Healthcare</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jBPM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tuning IOT-driven Camel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Programmers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Camel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Building deep learning XStream</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Artificial Intelligence, Security</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Financial services</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XStream</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Securing scalable Docker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jay Watt, Amy Fox</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Culture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Docker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Debug enterprise Hibernate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beth Green, Amy Cole</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hibernate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prepare for streaming GWT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beth Fox, Chad Green</t>
+    <t xml:space="preserve">Weld</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Troubleshooting reliable RestEasy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile, Culture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RestEasy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Using secure Android</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Android</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deliver stable Tensorflow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloud, Culture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tensorflow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implement platform-independent VertX</t>
   </si>
   <si>
     <t xml:space="preserve">Middleware</t>
   </si>
   <si>
-    <t xml:space="preserve">GWT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Understand mobile Errai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Errai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Applying modern Angular</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cloud, Middleware</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Angular</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grok distributed Weld</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flo Li, Gus Poe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mobile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weld</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Troubleshooting reliable RestEasy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Security</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RestEasy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Using secure Android</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ivy Smith, Jay Watt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Android</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deliver stable Tensorflow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tensorflow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implement platform-independent VertX</t>
-  </si>
-  <si>
     <t xml:space="preserve">VertX</t>
   </si>
   <si>
@@ -862,14 +868,14 @@
     <t xml:space="preserve">Total</t>
   </si>
   <si>
-    <t xml:space="preserve">S11: Understand mobile Errai
+    <t xml:space="preserve">S10: Prepare for streaming GWT
   Dan Jones</t>
   </si>
   <si>
     <t xml:space="preserve">Speaker</t>
   </si>
   <si>
-    <t xml:space="preserve">S11 @ R 1</t>
+    <t xml:space="preserve">S10 @ R 1</t>
   </si>
   <si>
     <t xml:space="preserve">Theme track tag</t>
@@ -887,7 +893,7 @@
     <t xml:space="preserve">Content tag</t>
   </si>
   <si>
-    <t xml:space="preserve">S11 (level 1)</t>
+    <t xml:space="preserve">S10 (level 1)</t>
   </si>
   <si>
     <t xml:space="preserve">Constraint match</t>
@@ -1520,25 +1526,25 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1564,7 +1570,7 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="13.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="8" style="0" width="8.67"/>
   </cols>
@@ -1582,34 +1588,34 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -1658,34 +1664,34 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -1734,34 +1740,34 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -1810,44 +1816,44 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -1882,13 +1888,13 @@
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -2041,14 +2047,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="4" style="0" width="13.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="10" style="0" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="5" style="0" width="13.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="11" style="0" width="8.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2069,13 +2076,13 @@
         <v>81</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>83</v>
@@ -2092,89 +2099,107 @@
       <c r="I2" s="1" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J2" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B3" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D3" s="2"/>
+      <c r="D3" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B4" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B5" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>630</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D5" s="2"/>
+      <c r="D5" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D6" s="2"/>
+      <c r="D6" s="2" t="s">
+        <v>94</v>
+      </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="B7" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>490</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D7" s="2"/>
+      <c r="D7" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2235,51 +2260,51 @@
         <v>81</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -2298,7 +2323,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -2317,16 +2342,14 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
-      <c r="G5" s="2" t="s">
-        <v>92</v>
-      </c>
+      <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -2338,7 +2361,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -2357,7 +2380,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2376,7 +2399,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2386,25 +2409,23 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
-      <c r="G9" s="2" t="s">
-        <v>92</v>
-      </c>
+      <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -2416,7 +2437,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2435,7 +2456,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -2445,25 +2466,23 @@
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
-      <c r="G12" s="2" t="s">
-        <v>92</v>
-      </c>
+      <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -2475,7 +2494,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -2494,7 +2513,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -2536,12 +2555,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="37.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="28.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="17.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="17.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="19.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="24.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="25.4"/>
@@ -2565,76 +2584,76 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="Y1" s="1" t="s">
         <v>64</v>
@@ -2643,39 +2662,37 @@
         <v>65</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>103</v>
+        <v>135</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>135</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="F2" s="2"/>
       <c r="G2" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -2688,10 +2705,10 @@
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
       <c r="U2" s="2" t="n">
-        <v>663</v>
+        <v>623</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W2" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -2704,32 +2721,34 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>104</v>
+        <v>142</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="F3" s="2"/>
+        <v>136</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>143</v>
+      </c>
       <c r="G3" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -2742,10 +2761,10 @@
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
       <c r="U3" s="2" t="n">
-        <v>474</v>
+        <v>291</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="W3" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -2758,32 +2777,32 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>146</v>
+        <v>108</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -2796,10 +2815,10 @@
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
       <c r="U4" s="2" t="n">
-        <v>362</v>
+        <v>214</v>
       </c>
       <c r="V4" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W4" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -2812,32 +2831,32 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -2850,10 +2869,10 @@
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
       <c r="U5" s="2" t="n">
-        <v>82</v>
+        <v>761</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W5" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -2864,36 +2883,34 @@
       <c r="Z5" s="2"/>
       <c r="AA5" s="2"/>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>108</v>
+        <v>157</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>135</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="F6" s="2"/>
       <c r="G6" s="2" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -2906,7 +2923,7 @@
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
       <c r="U6" s="2" t="n">
-        <v>841</v>
+        <v>388</v>
       </c>
       <c r="V6" s="2" t="n">
         <v>2</v>
@@ -2920,36 +2937,36 @@
       <c r="Z6" s="2"/>
       <c r="AA6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
@@ -2962,10 +2979,10 @@
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
       <c r="U7" s="2" t="n">
-        <v>957</v>
+        <v>798</v>
       </c>
       <c r="V7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W7" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -2976,34 +2993,36 @@
       <c r="Z7" s="2"/>
       <c r="AA7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="F8" s="2"/>
+        <v>148</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>166</v>
+      </c>
       <c r="G8" s="2" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
@@ -3016,10 +3035,10 @@
       <c r="S8" s="2"/>
       <c r="T8" s="2"/>
       <c r="U8" s="2" t="n">
-        <v>628</v>
+        <v>401</v>
       </c>
       <c r="V8" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="W8" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -3030,36 +3049,34 @@
       <c r="Z8" s="2"/>
       <c r="AA8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>111</v>
+        <v>170</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>168</v>
-      </c>
+        <v>171</v>
+      </c>
+      <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>1</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
@@ -3072,10 +3089,10 @@
       <c r="S9" s="2"/>
       <c r="T9" s="2"/>
       <c r="U9" s="2" t="n">
-        <v>509</v>
+        <v>720</v>
       </c>
       <c r="V9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W9" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -3086,34 +3103,34 @@
       <c r="Z9" s="2"/>
       <c r="AA9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>172</v>
+        <v>105</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
@@ -3126,10 +3143,10 @@
       <c r="S10" s="2"/>
       <c r="T10" s="2"/>
       <c r="U10" s="2" t="n">
-        <v>349</v>
+        <v>55</v>
       </c>
       <c r="V10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W10" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -3140,34 +3157,36 @@
       <c r="Z10" s="2"/>
       <c r="AA10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>177</v>
+        <v>106</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F11" s="2"/>
+        <v>179</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>180</v>
+      </c>
       <c r="G11" s="2" t="s">
-        <v>163</v>
+        <v>137</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
@@ -3180,10 +3199,10 @@
       <c r="S11" s="2"/>
       <c r="T11" s="2"/>
       <c r="U11" s="2" t="n">
-        <v>166</v>
+        <v>333</v>
       </c>
       <c r="V11" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W11" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -3194,34 +3213,34 @@
       <c r="Z11" s="2"/>
       <c r="AA11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>181</v>
+        <v>107</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
@@ -3234,48 +3253,58 @@
       <c r="S12" s="2"/>
       <c r="T12" s="2"/>
       <c r="U12" s="2" t="n">
-        <v>435</v>
+        <v>546</v>
       </c>
       <c r="V12" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="W12" s="2" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="X12" s="2"/>
-      <c r="Y12" s="2"/>
-      <c r="Z12" s="2"/>
-      <c r="AA12" s="2"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2</v>
+      </c>
+      <c r="W12" s="5" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="X12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y12" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="Z12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="AA12" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>106</v>
+        <v>187</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="F13" s="2"/>
+        <v>188</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>143</v>
+      </c>
       <c r="G13" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
@@ -3288,58 +3317,48 @@
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
       <c r="U13" s="2" t="n">
-        <v>429</v>
+        <v>785</v>
       </c>
       <c r="V13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="W13" s="2" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="W13" s="5" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="X13" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="Y13" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="Z13" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="AA13" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="X13" s="2"/>
+      <c r="Y13" s="2"/>
+      <c r="Z13" s="2"/>
+      <c r="AA13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>168</v>
-      </c>
+        <v>188</v>
+      </c>
+      <c r="F14" s="2"/>
       <c r="G14" s="2" t="s">
-        <v>163</v>
+        <v>144</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
@@ -3352,7 +3371,7 @@
       <c r="S14" s="2"/>
       <c r="T14" s="2"/>
       <c r="U14" s="2" t="n">
-        <v>340</v>
+        <v>245</v>
       </c>
       <c r="V14" s="2" t="n">
         <v>1</v>
@@ -3368,32 +3387,34 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>193</v>
+        <v>111</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="F15" s="2"/>
+        <v>195</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>162</v>
+      </c>
       <c r="G15" s="2" t="s">
-        <v>163</v>
+        <v>137</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -3406,10 +3427,10 @@
       <c r="S15" s="2"/>
       <c r="T15" s="2"/>
       <c r="U15" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="V15" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="V15" s="2" t="n">
-        <v>2</v>
       </c>
       <c r="W15" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -3422,32 +3443,32 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>3</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
@@ -3460,10 +3481,10 @@
       <c r="S16" s="2"/>
       <c r="T16" s="2"/>
       <c r="U16" s="2" t="n">
-        <v>957</v>
+        <v>318</v>
       </c>
       <c r="V16" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W16" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -3476,32 +3497,32 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>202</v>
+        <v>113</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>173</v>
+        <v>148</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>203</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
@@ -3514,10 +3535,10 @@
       <c r="S17" s="2"/>
       <c r="T17" s="2"/>
       <c r="U17" s="2" t="n">
-        <v>288</v>
+        <v>56</v>
       </c>
       <c r="V17" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W17" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -3539,23 +3560,23 @@
         <v>73</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -3568,7 +3589,7 @@
       <c r="S18" s="2"/>
       <c r="T18" s="2"/>
       <c r="U18" s="2" t="n">
-        <v>39</v>
+        <v>596</v>
       </c>
       <c r="V18" s="2" t="n">
         <v>3</v>
@@ -3584,32 +3605,32 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>177</v>
+        <v>115</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>173</v>
+        <v>210</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
@@ -3622,10 +3643,10 @@
       <c r="S19" s="2"/>
       <c r="T19" s="2"/>
       <c r="U19" s="2" t="n">
-        <v>458</v>
+        <v>701</v>
       </c>
       <c r="V19" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W19" s="2" t="n">
         <f aca="false">FALSE()</f>
@@ -3666,27 +3687,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3725,7 +3746,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>18</v>
@@ -3778,34 +3799,34 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="4"/>
@@ -3814,7 +3835,7 @@
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="2"/>
@@ -3825,7 +3846,7 @@
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="2"/>
@@ -3847,7 +3868,7 @@
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="4"/>
@@ -3898,30 +3919,30 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -3932,7 +3953,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -3943,7 +3964,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -3954,11 +3975,11 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -3967,7 +3988,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3978,18 +3999,18 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
+        <v>109</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -4000,7 +4021,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -4011,18 +4032,18 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+        <v>112</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -4033,7 +4054,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -4044,7 +4065,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -4077,7 +4098,7 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="13.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="8" style="0" width="8.67"/>
   </cols>
@@ -4095,34 +4116,34 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>154</v>
+        <v>179</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>

</xml_diff>

<commit_message>
Change tag to tags in rules and genereate new example xlsx files
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -36,6 +36,8 @@
         <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
+-10soft total
+    -10soft for 1 Crowd controls
 </t>
       </text>
     </comment>
@@ -54,6 +56,8 @@
         <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
+-10soft total
+    -10soft for 1 Crowd controls
 </t>
       </text>
     </comment>
@@ -72,6 +76,8 @@
         <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
+-10soft total
+    -10soft for 1 Crowd controls
 </t>
       </text>
     </comment>
@@ -90,6 +96,8 @@
         <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
+-10soft total
+    -10soft for 1 Crowd controls
 </t>
       </text>
     </comment>
@@ -108,6 +116,8 @@
         <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
+-10soft total
+    -10soft for 1 Crowd controls
 </t>
       </text>
     </comment>
@@ -126,6 +136,8 @@
         <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
+-10soft total
+    -10soft for 1 Crowd controls
 </t>
       </text>
     </comment>
@@ -144,6 +156,8 @@
         <t xml:space="preserve">S10: Prepare for streaming GWT
     Dan Jones
 PINNED BY USER
+-10soft total
+    -10soft for 1 Crowd controls
 </t>
       </text>
     </comment>
@@ -152,7 +166,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="238">
   <si>
     <t>Conference name</t>
   </si>
@@ -265,6 +279,12 @@
     <t>Soft penalty per 2 talks where the less popular one (has lower number of likes) is assigned a larger room than the more popular talk</t>
   </si>
   <si>
+    <t>Crowd control</t>
+  </si>
+  <si>
+    <t>Soft penalty per talks with crowd control risk greater than zero that are not in pairs</t>
+  </si>
+  <si>
     <t>Talk type of timeslot</t>
   </si>
   <si>
@@ -802,7 +822,7 @@
     <t>Score</t>
   </si>
   <si>
-    <t>-34init</t>
+    <t>-34init/-10soft</t>
   </si>
   <si>
     <t>Count</t>
@@ -855,6 +875,12 @@
   </si>
   <si>
     <t>Total score</t>
+  </si>
+  <si>
+    <t>-10soft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    S10</t>
   </si>
 </sst>
 </file>
@@ -1242,18 +1268,18 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="1" t="s">
+    <row r="22">
+      <c r="A22" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="2" t="n">
-        <v>10000.0</v>
-      </c>
-      <c r="C23" s="1" t="s">
+      <c r="B22" s="2" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>38</v>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="1" t="s">
         <v>39</v>
@@ -1281,7 +1307,7 @@
         <v>43</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>10.0</v>
+        <v>10000.0</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>44</v>
@@ -1292,7 +1318,7 @@
         <v>45</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>1.0</v>
+        <v>10.0</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>46</v>
@@ -1339,12 +1365,12 @@
         <v>1.0</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>1.0</v>
@@ -1355,13 +1381,13 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34">
@@ -1383,12 +1409,12 @@
         <v>1.0</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>1.0</v>
@@ -1399,13 +1425,13 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38">
@@ -1417,6 +1443,17 @@
       </c>
       <c r="C38" s="1" t="s">
         <v>64</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1444,48 +1481,48 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1516,71 +1553,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1612,71 +1649,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1708,71 +1745,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1804,77 +1841,77 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -1903,14 +1940,33 @@
     <row r="1"/>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>233</v>
-      </c>
+        <v>235</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -1932,121 +1988,121 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -2074,226 +2130,226 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>60.0</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>240.0</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>630.0</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>70.0</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>490.0</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -2329,660 +2385,660 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -3030,147 +3086,147 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U2" s="2" t="n">
         <v>623.0</v>
@@ -3182,78 +3238,78 @@
         <v>0</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA2" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U3" s="2" t="n">
         <v>291.0</v>
@@ -3265,78 +3321,78 @@
         <v>0</v>
       </c>
       <c r="X3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U4" s="2" t="n">
         <v>214.0</v>
@@ -3348,78 +3404,78 @@
         <v>0</v>
       </c>
       <c r="X4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA4" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U5" s="2" t="n">
         <v>761.0</v>
@@ -3431,78 +3487,78 @@
         <v>0</v>
       </c>
       <c r="X5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA5" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U6" s="2" t="n">
         <v>388.0</v>
@@ -3514,78 +3570,78 @@
         <v>0</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA6" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U7" s="2" t="n">
         <v>798.0</v>
@@ -3597,78 +3653,78 @@
         <v>0</v>
       </c>
       <c r="X7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA7" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U8" s="2" t="n">
         <v>401.0</v>
@@ -3680,78 +3736,78 @@
         <v>0</v>
       </c>
       <c r="X8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U9" s="2" t="n">
         <v>720.0</v>
@@ -3763,78 +3819,78 @@
         <v>0</v>
       </c>
       <c r="X9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA9" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U10" s="2" t="n">
         <v>55.0</v>
@@ -3846,78 +3902,78 @@
         <v>0</v>
       </c>
       <c r="X10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA10" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U11" s="2" t="n">
         <v>333.0</v>
@@ -3929,78 +3985,78 @@
         <v>0</v>
       </c>
       <c r="X11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA11" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U12" s="2" t="n">
         <v>546.0</v>
@@ -4012,78 +4068,78 @@
         <v>1</v>
       </c>
       <c r="X12" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="Y12" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Z12" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="AA12" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U13" s="2" t="n">
         <v>785.0</v>
@@ -4095,78 +4151,78 @@
         <v>0</v>
       </c>
       <c r="X13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA13" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>191</v>
-      </c>
       <c r="F14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U14" s="2" t="n">
         <v>245.0</v>
@@ -4178,78 +4234,78 @@
         <v>0</v>
       </c>
       <c r="X14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA14" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U15" s="2" t="n">
         <v>156.0</v>
@@ -4261,78 +4317,78 @@
         <v>0</v>
       </c>
       <c r="X15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA15" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U16" s="2" t="n">
         <v>318.0</v>
@@ -4344,78 +4400,78 @@
         <v>0</v>
       </c>
       <c r="X16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA16" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U17" s="2" t="n">
         <v>56.0</v>
@@ -4427,78 +4483,78 @@
         <v>0</v>
       </c>
       <c r="X17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U18" s="2" t="n">
         <v>596.0</v>
@@ -4510,78 +4566,78 @@
         <v>0</v>
       </c>
       <c r="X18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="R19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="S19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="T19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U19" s="2" t="n">
         <v>701.0</v>
@@ -4593,16 +4649,16 @@
         <v>0</v>
       </c>
       <c r="X19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Y19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AA19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -4620,7 +4676,7 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="10.78515625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="7.27734375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="13.98828125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="18.4296875" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="15.25" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="17.625" customWidth="true" bestFit="true"/>
@@ -4628,33 +4684,33 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>2.0</v>
@@ -4671,7 +4727,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>16.0</v>
@@ -4689,7 +4745,7 @@
     <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>18.0</v>
@@ -4736,163 +4792,163 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" ht="45.0" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" ht="45.0" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" ht="45.0" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" ht="45.0" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" ht="45.0" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -4931,324 +4987,324 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" ht="15.0" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="true">
       <c r="A8" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="true">
       <c r="A9" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" ht="15.0" customHeight="true">
       <c r="A10" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" ht="15.0" customHeight="true">
       <c r="A11" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="true">
       <c r="A12" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13" ht="15.0" customHeight="true">
       <c r="A13" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" ht="15.0" customHeight="true">
       <c r="A14" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -5280,71 +5336,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Generate new files with new constraint
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -181,7 +181,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1207" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="251">
   <si>
     <t>Conference name</t>
   </si>
@@ -400,6 +400,12 @@
   </si>
   <si>
     <t>Hard penalty per talk that is scheduled before any of its prerequisite talks</t>
+  </si>
+  <si>
+    <t>Consecutive talks pause</t>
+  </si>
+  <si>
+    <t>Hard penalty per two consecutive talks for the same speaker with a pause less than minimum pause</t>
   </si>
   <si>
     <t>Day</t>
@@ -1162,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="43.66796875" customWidth="true" bestFit="true"/>
@@ -1608,6 +1614,17 @@
       </c>
       <c r="C43" s="1" t="s">
         <v>72</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1635,48 +1652,48 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1707,71 +1724,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1803,71 +1820,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1899,71 +1916,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1995,71 +2012,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -2087,22 +2104,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4">
@@ -2111,15 +2128,15 @@
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -2144,58 +2161,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" ht="45.0" customHeight="true">
       <c r="A2" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" ht="45.0" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" ht="45.0" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" ht="45.0" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" ht="45.0" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" ht="45.0" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -2219,121 +2236,121 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -2361,226 +2378,226 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>60.0</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>240.0</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>630.0</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>70.0</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>490.0</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -2616,660 +2633,660 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -3321,159 +3338,159 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U2" s="2" t="n">
         <v>623.0</v>
@@ -3485,90 +3502,90 @@
         <v>0</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE2" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U3" s="2" t="n">
         <v>291.0</v>
@@ -3580,90 +3597,90 @@
         <v>0</v>
       </c>
       <c r="X3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE3" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U4" s="2" t="n">
         <v>214.0</v>
@@ -3675,90 +3692,90 @@
         <v>0</v>
       </c>
       <c r="X4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE4" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U5" s="2" t="n">
         <v>761.0</v>
@@ -3770,90 +3787,90 @@
         <v>0</v>
       </c>
       <c r="X5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE5" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U6" s="2" t="n">
         <v>388.0</v>
@@ -3865,90 +3882,90 @@
         <v>0</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE6" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U7" s="2" t="n">
         <v>798.0</v>
@@ -3960,90 +3977,90 @@
         <v>0</v>
       </c>
       <c r="X7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE7" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U8" s="2" t="n">
         <v>401.0</v>
@@ -4055,90 +4072,90 @@
         <v>0</v>
       </c>
       <c r="X8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE8" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U9" s="2" t="n">
         <v>720.0</v>
@@ -4150,90 +4167,90 @@
         <v>0</v>
       </c>
       <c r="X9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE9" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U10" s="2" t="n">
         <v>55.0</v>
@@ -4245,90 +4262,90 @@
         <v>0</v>
       </c>
       <c r="X10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE10" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U11" s="2" t="n">
         <v>333.0</v>
@@ -4340,90 +4357,90 @@
         <v>0</v>
       </c>
       <c r="X11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE11" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U12" s="2" t="n">
         <v>546.0</v>
@@ -4435,90 +4452,90 @@
         <v>1</v>
       </c>
       <c r="X12" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="Y12" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="Z12" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AA12" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="AB12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE12" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U13" s="2" t="n">
         <v>785.0</v>
@@ -4530,90 +4547,90 @@
         <v>0</v>
       </c>
       <c r="X13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE13" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>203</v>
-      </c>
       <c r="F14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U14" s="2" t="n">
         <v>245.0</v>
@@ -4625,90 +4642,90 @@
         <v>0</v>
       </c>
       <c r="X14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE14" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U15" s="2" t="n">
         <v>156.0</v>
@@ -4720,90 +4737,90 @@
         <v>0</v>
       </c>
       <c r="X15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE15" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U16" s="2" t="n">
         <v>318.0</v>
@@ -4815,90 +4832,90 @@
         <v>0</v>
       </c>
       <c r="X16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE16" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U17" s="2" t="n">
         <v>56.0</v>
@@ -4910,90 +4927,90 @@
         <v>0</v>
       </c>
       <c r="X17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE17" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U18" s="2" t="n">
         <v>596.0</v>
@@ -5005,90 +5022,90 @@
         <v>0</v>
       </c>
       <c r="X18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE18" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="R19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="T19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U19" s="2" t="n">
         <v>701.0</v>
@@ -5100,28 +5117,28 @@
         <v>0</v>
       </c>
       <c r="X19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Y19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="Z19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AA19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AB19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AD19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AE19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -5147,33 +5164,33 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>2.0</v>
@@ -5190,7 +5207,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>16.0</v>
@@ -5208,7 +5225,7 @@
     <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>18.0</v>
@@ -5255,163 +5272,163 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" ht="45.0" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" ht="45.0" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" ht="45.0" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" ht="45.0" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" ht="45.0" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -5450,324 +5467,324 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" ht="15.0" customHeight="true">
       <c r="A4" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="true">
       <c r="A6" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" ht="15.0" customHeight="true">
       <c r="A7" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="true">
       <c r="A8" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" ht="15.0" customHeight="true">
       <c r="A9" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" ht="15.0" customHeight="true">
       <c r="A10" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" ht="15.0" customHeight="true">
       <c r="A11" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" ht="15.0" customHeight="true">
       <c r="A12" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" ht="15.0" customHeight="true">
       <c r="A13" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" ht="15.0" customHeight="true">
       <c r="A14" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -5799,71 +5816,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sonarcloud: fix a number of reported issues + disable crowd control in generated conf scheduling to generate solvable solutions
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -34,10 +34,9 @@
   <commentList>
     <comment ref="C3" authorId="0">
       <text>
-        <t xml:space="preserve">S10-Culture: Prepare for streaming GWT
-    Dan Jones
+        <t xml:space="preserve">S04-Security: Discover AI-driven OptaPlanner
+    Hugo Rye
 PINNED BY USER
--45hard total
 </t>
       </text>
     </comment>
@@ -53,10 +52,9 @@
   <commentList>
     <comment ref="C3" authorId="0">
       <text>
-        <t xml:space="preserve">S10-Culture: Prepare for streaming GWT
-    Dan Jones
+        <t xml:space="preserve">S04-Security: Discover AI-driven OptaPlanner
+    Hugo Rye
 PINNED BY USER
--45hard total
 </t>
       </text>
     </comment>
@@ -72,10 +70,9 @@
   <commentList>
     <comment ref="C3" authorId="0">
       <text>
-        <t xml:space="preserve">S10-Culture: Prepare for streaming GWT
-    Dan Jones
+        <t xml:space="preserve">S04-Security: Discover AI-driven OptaPlanner
+    Hugo Rye
 PINNED BY USER
--45hard total
 </t>
       </text>
     </comment>
@@ -91,10 +88,9 @@
   <commentList>
     <comment ref="C3" authorId="0">
       <text>
-        <t xml:space="preserve">S10-Culture: Prepare for streaming GWT
-    Dan Jones
+        <t xml:space="preserve">S04-Security: Discover AI-driven OptaPlanner
+    Hugo Rye
 PINNED BY USER
--45hard total
 </t>
       </text>
     </comment>
@@ -110,11 +106,9 @@
   <commentList>
     <comment ref="B3" authorId="0">
       <text>
-        <t xml:space="preserve">S10-Culture: Prepare for streaming GWT
-    Dan Jones
+        <t xml:space="preserve">S04-Security: Discover AI-driven OptaPlanner
+    Hugo Rye
 PINNED BY USER
--45hard total
-    -45hard for 1 Crowd controls
 </t>
       </text>
     </comment>
@@ -130,11 +124,9 @@
   <commentList>
     <comment ref="C3" authorId="0">
       <text>
-        <t xml:space="preserve">S10-Culture: Prepare for streaming GWT
-    Dan Jones
+        <t xml:space="preserve">S04-Security: Discover AI-driven OptaPlanner
+    Hugo Rye
 PINNED BY USER
--45hard total
-    -45hard for 1 Crowd controls
 </t>
       </text>
     </comment>
@@ -148,12 +140,11 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="C6" authorId="0">
+    <comment ref="C10" authorId="0">
       <text>
-        <t xml:space="preserve">S10-Culture: Prepare for streaming GWT
-    Dan Jones
+        <t xml:space="preserve">S04-Security: Discover AI-driven OptaPlanner
+    Hugo Rye
 PINNED BY USER
--45hard total
 </t>
       </text>
     </comment>
@@ -169,10 +160,9 @@
   <commentList>
     <comment ref="C3" authorId="0">
       <text>
-        <t xml:space="preserve">S10-Culture: Prepare for streaming GWT
-    Dan Jones
+        <t xml:space="preserve">S04-Security: Discover AI-driven OptaPlanner
+    Hugo Rye
 PINNED BY USER
--45hard total
 </t>
       </text>
     </comment>
@@ -181,7 +171,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1469" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1467" uniqueCount="270">
   <si>
     <t>Conference name</t>
   </si>
@@ -687,189 +677,189 @@
     <t>Advanced containerized WildFly</t>
   </si>
   <si>
-    <t>Chad Green, Dan Jones</t>
+    <t>Chad Green, Dan Jones, Elsa King</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>WildFly</t>
+  </si>
+  <si>
+    <t>S02</t>
+  </si>
+  <si>
+    <t>Learn virtualized Spring</t>
+  </si>
+  <si>
+    <t>Culture</t>
+  </si>
+  <si>
+    <t>Spring</t>
+  </si>
+  <si>
+    <t>S03</t>
+  </si>
+  <si>
+    <t>Intro to serverless Drools</t>
+  </si>
+  <si>
+    <t>Drools</t>
+  </si>
+  <si>
+    <t>S04</t>
+  </si>
+  <si>
+    <t>Discover AI-driven OptaPlanner</t>
+  </si>
+  <si>
+    <t>Managers</t>
+  </si>
+  <si>
+    <t>OptaPlanner</t>
+  </si>
+  <si>
+    <t>S05</t>
+  </si>
+  <si>
+    <t>Mastering machine learning jBPM</t>
+  </si>
+  <si>
+    <t>jBPM</t>
+  </si>
+  <si>
+    <t>S06</t>
+  </si>
+  <si>
+    <t>Tuning IOT-driven Camel</t>
+  </si>
+  <si>
+    <t>Jay Watt, Amy Fox</t>
+  </si>
+  <si>
+    <t>Modern Web</t>
+  </si>
+  <si>
+    <t>Camel</t>
+  </si>
+  <si>
+    <t>S07</t>
+  </si>
+  <si>
+    <t>Building deep learning XStream</t>
+  </si>
+  <si>
+    <t>Artificial Intelligence</t>
+  </si>
+  <si>
+    <t>Programmers</t>
+  </si>
+  <si>
+    <t>XStream</t>
+  </si>
+  <si>
+    <t>S08</t>
+  </si>
+  <si>
+    <t>Securing scalable Docker</t>
+  </si>
+  <si>
+    <t>Amy Cole, Beth Fox, Chad Green</t>
   </si>
   <si>
     <t>Transportation</t>
   </si>
   <si>
-    <t>Managers</t>
-  </si>
-  <si>
-    <t>WildFly</t>
-  </si>
-  <si>
-    <t>S02</t>
-  </si>
-  <si>
-    <t>Learn virtualized Spring</t>
+    <t>Docker</t>
+  </si>
+  <si>
+    <t>S09</t>
+  </si>
+  <si>
+    <t>Debug enterprise Hibernate</t>
+  </si>
+  <si>
+    <t>Hibernate</t>
+  </si>
+  <si>
+    <t>S10</t>
+  </si>
+  <si>
+    <t>Prepare for streaming GWT</t>
+  </si>
+  <si>
+    <t>Elsa King, Flo Li</t>
+  </si>
+  <si>
+    <t>GWT</t>
+  </si>
+  <si>
+    <t>S11</t>
+  </si>
+  <si>
+    <t>Understand mobile Errai</t>
+  </si>
+  <si>
+    <t>Modern Web, Security</t>
+  </si>
+  <si>
+    <t>Errai</t>
+  </si>
+  <si>
+    <t>S12</t>
+  </si>
+  <si>
+    <t>Applying modern Angular</t>
+  </si>
+  <si>
+    <t>Hugo Rye, Ivy Smith</t>
   </si>
   <si>
     <t>IoT</t>
   </si>
   <si>
-    <t>Programmers</t>
-  </si>
-  <si>
-    <t>Spring</t>
-  </si>
-  <si>
-    <t>S03</t>
-  </si>
-  <si>
-    <t>Intro to serverless Drools</t>
-  </si>
-  <si>
-    <t>Big Data, Culture</t>
-  </si>
-  <si>
-    <t>Drools</t>
-  </si>
-  <si>
-    <t>S04</t>
-  </si>
-  <si>
-    <t>Discover AI-driven OptaPlanner</t>
-  </si>
-  <si>
-    <t>Gus Poe, Hugo Rye</t>
-  </si>
-  <si>
-    <t>OptaPlanner</t>
-  </si>
-  <si>
-    <t>S05</t>
-  </si>
-  <si>
-    <t>Mastering machine learning jBPM</t>
-  </si>
-  <si>
-    <t>Middleware, Modern Web</t>
+    <t>Angular</t>
+  </si>
+  <si>
+    <t>S13</t>
+  </si>
+  <si>
+    <t>Grok distributed Weld</t>
+  </si>
+  <si>
+    <t>Cloud, Middleware</t>
   </si>
   <si>
     <t>Financial services</t>
   </si>
   <si>
-    <t>jBPM</t>
-  </si>
-  <si>
-    <t>S06</t>
-  </si>
-  <si>
-    <t>Tuning IOT-driven Camel</t>
-  </si>
-  <si>
-    <t>Government</t>
-  </si>
-  <si>
-    <t>Camel</t>
-  </si>
-  <si>
-    <t>S07</t>
-  </si>
-  <si>
-    <t>Building deep learning XStream</t>
-  </si>
-  <si>
-    <t>Amy Fox, Beth Green, Amy Cole</t>
+    <t>Weld</t>
+  </si>
+  <si>
+    <t>S14</t>
+  </si>
+  <si>
+    <t>Troubleshooting reliable RestEasy</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>RestEasy</t>
+  </si>
+  <si>
+    <t>S15</t>
+  </si>
+  <si>
+    <t>Using secure Android</t>
   </si>
   <si>
     <t>Cloud</t>
   </si>
   <si>
-    <t>XStream</t>
-  </si>
-  <si>
-    <t>S08</t>
-  </si>
-  <si>
-    <t>Securing scalable Docker</t>
-  </si>
-  <si>
-    <t>Security, Culture</t>
-  </si>
-  <si>
-    <t>Docker, Kubernetes</t>
-  </si>
-  <si>
-    <t>S09</t>
-  </si>
-  <si>
-    <t>Debug enterprise Hibernate</t>
-  </si>
-  <si>
-    <t>Culture</t>
-  </si>
-  <si>
-    <t>Telecommunications</t>
-  </si>
-  <si>
-    <t>Hibernate</t>
-  </si>
-  <si>
-    <t>S10</t>
-  </si>
-  <si>
-    <t>Prepare for streaming GWT</t>
-  </si>
-  <si>
-    <t>GWT</t>
-  </si>
-  <si>
-    <t>S11</t>
-  </si>
-  <si>
-    <t>Understand mobile Errai</t>
-  </si>
-  <si>
-    <t>Elsa King, Flo Li</t>
-  </si>
-  <si>
-    <t>Artificial Intelligence</t>
-  </si>
-  <si>
-    <t>Errai</t>
-  </si>
-  <si>
-    <t>S12</t>
-  </si>
-  <si>
-    <t>Applying modern Angular</t>
-  </si>
-  <si>
-    <t>Angular</t>
-  </si>
-  <si>
-    <t>S13</t>
-  </si>
-  <si>
-    <t>Grok distributed Weld</t>
-  </si>
-  <si>
-    <t>Middleware, Security</t>
-  </si>
-  <si>
-    <t>Weld</t>
-  </si>
-  <si>
-    <t>S14</t>
-  </si>
-  <si>
-    <t>Troubleshooting reliable RestEasy</t>
-  </si>
-  <si>
-    <t>Mobile, Culture</t>
-  </si>
-  <si>
-    <t>RestEasy</t>
-  </si>
-  <si>
-    <t>S15</t>
-  </si>
-  <si>
-    <t>Using secure Android</t>
-  </si>
-  <si>
     <t>Android</t>
   </si>
   <si>
@@ -879,9 +869,6 @@
     <t>Deliver stable Tensorflow</t>
   </si>
   <si>
-    <t>Cloud, Culture</t>
-  </si>
-  <si>
     <t>Tensorflow</t>
   </si>
   <si>
@@ -891,16 +878,13 @@
     <t>Implement platform-independent VertX</t>
   </si>
   <si>
-    <t>Middleware</t>
-  </si>
-  <si>
     <t>VertX</t>
   </si>
   <si>
     <t>Score</t>
   </si>
   <si>
-    <t>-34init/-45hard</t>
+    <t>-34init</t>
   </si>
   <si>
     <t>Count</t>
@@ -918,14 +902,14 @@
     <t>Total</t>
   </si>
   <si>
-    <t>S10: Prepare for streaming GWT
-  Dan Jones</t>
+    <t>S04: Discover AI-driven OptaPlanner
+  Hugo Rye</t>
   </si>
   <si>
     <t>Speaker</t>
   </si>
   <si>
-    <t>S10 @ R 1</t>
+    <t>S04 @ R 1</t>
   </si>
   <si>
     <t>Theme track tag</t>
@@ -937,13 +921,13 @@
     <t>Audience type</t>
   </si>
   <si>
-    <t>1</t>
+    <t>3</t>
   </si>
   <si>
     <t>Content tag</t>
   </si>
   <si>
-    <t>S10 (level 1)</t>
+    <t>S04 (level 3)</t>
   </si>
   <si>
     <t>Constraint name</t>
@@ -982,9 +966,6 @@
     <t>1hard</t>
   </si>
   <si>
-    <t>-45hard</t>
-  </si>
-  <si>
     <t>1medium</t>
   </si>
   <si>
@@ -1000,8 +981,8 @@
     <t>1soft</t>
   </si>
   <si>
-    <t>Prepare for streaming GWT
-Dan Jones</t>
+    <t>Discover AI-driven OptaPlanner
+Hugo Rye</t>
   </si>
 </sst>
 </file>
@@ -1749,7 +1730,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>105</v>
@@ -1821,7 +1802,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>105</v>
@@ -1844,13 +1825,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>93</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>93</v>
@@ -1940,13 +1921,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>93</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>93</v>
@@ -1979,7 +1960,7 @@
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="11.78515625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="12.62109375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="11.86328125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="11.9140625" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="11.86328125" customWidth="true" bestFit="true"/>
@@ -2013,7 +1994,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>105</v>
@@ -2036,13 +2017,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>210</v>
+        <v>181</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>93</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>93</v>
@@ -2138,7 +2119,7 @@
         <v>93</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>93</v>
@@ -2168,13 +2149,13 @@
   <sheetPr>
     <tabColor rgb="FCE94F"/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="17.34375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="12.65234375" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="8.0703125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="6.0859375" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="1.0546875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="12.296875" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="12.9296875" customWidth="true" bestFit="true"/>
@@ -2182,39 +2163,39 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="D3" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>256</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -2227,13 +2208,13 @@
         <v>7</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6">
@@ -2241,13 +2222,13 @@
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7">
@@ -2255,13 +2236,13 @@
         <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8">
@@ -2269,13 +2250,13 @@
         <v>16</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="9">
@@ -2283,13 +2264,13 @@
         <v>19</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="10">
@@ -2297,13 +2278,13 @@
         <v>24</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11">
@@ -2311,13 +2292,13 @@
         <v>26</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12">
@@ -2325,13 +2306,13 @@
         <v>36</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="13">
@@ -2339,13 +2320,13 @@
         <v>30</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14">
@@ -2353,13 +2334,13 @@
         <v>34</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C14" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15">
@@ -2367,13 +2348,13 @@
         <v>28</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="16">
@@ -2381,13 +2362,13 @@
         <v>21</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17">
@@ -2395,13 +2376,13 @@
         <v>39</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="18">
@@ -2409,13 +2390,13 @@
         <v>33</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C18" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="19">
@@ -2423,13 +2404,13 @@
         <v>38</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C19" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="20">
@@ -2437,13 +2418,13 @@
         <v>32</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C20" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="21">
@@ -2451,13 +2432,13 @@
         <v>40</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C21" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="22">
@@ -2465,13 +2446,13 @@
         <v>62</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C22" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="23">
@@ -2479,13 +2460,13 @@
         <v>78</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C23" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="24">
@@ -2493,13 +2474,13 @@
         <v>71</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C24" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="25">
@@ -2507,13 +2488,13 @@
         <v>80</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C25" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="26">
@@ -2521,13 +2502,13 @@
         <v>74</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C26" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="27">
@@ -2535,13 +2516,13 @@
         <v>82</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C27" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="28">
@@ -2549,13 +2530,13 @@
         <v>76</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C28" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="29">
@@ -2563,13 +2544,13 @@
         <v>83</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C29" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="30">
@@ -2577,13 +2558,13 @@
         <v>77</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C30" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="31">
@@ -2591,13 +2572,13 @@
         <v>60</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C31" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="32">
@@ -2605,13 +2586,13 @@
         <v>65</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C32" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="33">
@@ -2619,13 +2600,13 @@
         <v>69</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C33" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="34">
@@ -2633,13 +2614,13 @@
         <v>43</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C34" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="35">
@@ -2647,13 +2628,13 @@
         <v>67</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C35" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="36">
@@ -2661,13 +2642,13 @@
         <v>50</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C36" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="37">
@@ -2675,13 +2656,13 @@
         <v>46</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C37" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="38">
@@ -2689,13 +2670,13 @@
         <v>48</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C38" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="39">
@@ -2703,13 +2684,13 @@
         <v>58</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C39" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="40">
@@ -2717,13 +2698,13 @@
         <v>52</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C40" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="41">
@@ -2731,89 +2712,90 @@
         <v>55</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C41" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="42"/>
     <row r="43"/>
     <row r="44">
       <c r="A44" s="1" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>208</v>
+      <c r="A45" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="C46" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="C47" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="C48" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>265</v>
@@ -2822,455 +2804,441 @@
         <v>0.0</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="s">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="C50" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C51" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C52" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="s">
-        <v>69</v>
+        <v>43</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C53" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="C54" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="C55" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C56" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="C57" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C58" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="C59" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="s">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C60" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C61" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="s">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="C62" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C63" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C64" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C65" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="C66" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C67" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C68" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="C69" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="s">
-        <v>21</v>
+        <v>82</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C70" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C71" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="s">
-        <v>76</v>
+        <v>19</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="C72" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C73" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C74" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C75" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C76" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="s">
-        <v>32</v>
+        <v>83</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C77" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C78" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="s">
-        <v>77</v>
+        <v>46</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C79" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C80" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="C81" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="D81" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>
@@ -3311,8 +3279,8 @@
       <c r="A3" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>272</v>
+      <c r="B3" s="13" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="4" ht="45.0" customHeight="true">
@@ -4438,12 +4406,12 @@
     <col min="1" max="1" width="5.69140625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="36.7734375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="9.41796875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="29.4140625" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="24.78515625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="19.625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="30.52734375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="21.19921875" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="16.515625" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="16.4453125" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="14.4375" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="18.64453125" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="12.6640625" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="9.7109375" customWidth="true" bestFit="true"/>
     <col min="11" max="11" width="21.69921875" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="22.09765625" customWidth="true" bestFit="true"/>
@@ -4628,7 +4596,7 @@
         <v>623.0</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="W2" s="2" t="b">
         <v>0</v>
@@ -4672,19 +4640,19 @@
         <v>168</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>169</v>
+        <v>93</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>3.0</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>165</v>
@@ -4720,7 +4688,7 @@
         <v>93</v>
       </c>
       <c r="U3" s="2" t="n">
-        <v>291.0</v>
+        <v>942.0</v>
       </c>
       <c r="V3" s="2" t="n">
         <v>0.0</v>
@@ -4755,31 +4723,31 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>173</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>174</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>3.0</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>176</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>165</v>
@@ -4815,7 +4783,7 @@
         <v>93</v>
       </c>
       <c r="U4" s="2" t="n">
-        <v>214.0</v>
+        <v>293.0</v>
       </c>
       <c r="V4" s="2" t="n">
         <v>0.0</v>
@@ -4850,31 +4818,31 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>179</v>
+        <v>162</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>93</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>165</v>
@@ -4910,10 +4878,10 @@
         <v>93</v>
       </c>
       <c r="U5" s="2" t="n">
-        <v>761.0</v>
+        <v>82.0</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="W5" s="2" t="b">
         <v>0</v>
@@ -4945,31 +4913,31 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>183</v>
+        <v>133</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>93</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>165</v>
@@ -5005,25 +4973,25 @@
         <v>93</v>
       </c>
       <c r="U6" s="2" t="n">
-        <v>388.0</v>
+        <v>579.0</v>
       </c>
       <c r="V6" s="2" t="n">
-        <v>2.0</v>
-      </c>
-      <c r="W6" s="2" t="b">
-        <v>0</v>
+        <v>0.0</v>
+      </c>
+      <c r="W6" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="Y6" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="Z6" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AA6" s="2" t="s">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="AB6" s="2" t="s">
         <v>93</v>
@@ -5040,10 +5008,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>95</v>
@@ -5052,19 +5020,19 @@
         <v>134</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>188</v>
+        <v>93</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>165</v>
@@ -5100,10 +5068,10 @@
         <v>93</v>
       </c>
       <c r="U7" s="2" t="n">
-        <v>798.0</v>
+        <v>377.0</v>
       </c>
       <c r="V7" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="W7" s="2" t="b">
         <v>0</v>
@@ -5135,31 +5103,31 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>135</v>
+        <v>187</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>192</v>
+        <v>93</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>165</v>
@@ -5195,10 +5163,10 @@
         <v>93</v>
       </c>
       <c r="U8" s="2" t="n">
-        <v>401.0</v>
+        <v>196.0</v>
       </c>
       <c r="V8" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="W8" s="2" t="b">
         <v>0</v>
@@ -5230,31 +5198,31 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>196</v>
+        <v>137</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>93</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>165</v>
@@ -5290,10 +5258,10 @@
         <v>93</v>
       </c>
       <c r="U9" s="2" t="n">
-        <v>720.0</v>
+        <v>401.0</v>
       </c>
       <c r="V9" s="2" t="n">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="W9" s="2" t="b">
         <v>0</v>
@@ -5325,31 +5293,31 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>127</v>
+        <v>197</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>201</v>
+        <v>169</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>93</v>
+        <v>198</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>165</v>
@@ -5385,10 +5353,10 @@
         <v>93</v>
       </c>
       <c r="U10" s="2" t="n">
-        <v>55.0</v>
+        <v>226.0</v>
       </c>
       <c r="V10" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="W10" s="2" t="b">
         <v>0</v>
@@ -5420,31 +5388,31 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>205</v>
+        <v>169</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>206</v>
+        <v>93</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>163</v>
+        <v>193</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>165</v>
@@ -5480,7 +5448,7 @@
         <v>93</v>
       </c>
       <c r="U11" s="2" t="n">
-        <v>333.0</v>
+        <v>361.0</v>
       </c>
       <c r="V11" s="2" t="n">
         <v>0.0</v>
@@ -5515,31 +5483,31 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>129</v>
+        <v>205</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>205</v>
+        <v>169</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>93</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>165</v>
@@ -5575,25 +5543,25 @@
         <v>93</v>
       </c>
       <c r="U12" s="2" t="n">
-        <v>546.0</v>
+        <v>526.0</v>
       </c>
       <c r="V12" s="2" t="n">
-        <v>2.0</v>
-      </c>
-      <c r="W12" s="6" t="b">
-        <v>1</v>
+        <v>0.0</v>
+      </c>
+      <c r="W12" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="X12" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="Y12" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="Z12" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="AA12" s="2" t="s">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="AB12" s="2" t="s">
         <v>93</v>
@@ -5610,31 +5578,31 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>213</v>
+        <v>132</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>169</v>
+        <v>93</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>163</v>
+        <v>193</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>165</v>
@@ -5670,10 +5638,10 @@
         <v>93</v>
       </c>
       <c r="U13" s="2" t="n">
-        <v>785.0</v>
+        <v>185.0</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="W13" s="2" t="b">
         <v>0</v>
@@ -5705,16 +5673,16 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>132</v>
+        <v>213</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>214</v>
@@ -5723,13 +5691,13 @@
         <v>93</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>165</v>
@@ -5765,10 +5733,10 @@
         <v>93</v>
       </c>
       <c r="U14" s="2" t="n">
-        <v>245.0</v>
+        <v>405.0</v>
       </c>
       <c r="V14" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="W14" s="2" t="b">
         <v>0</v>
@@ -5800,31 +5768,31 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>188</v>
+        <v>219</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>163</v>
+        <v>193</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>165</v>
@@ -5860,10 +5828,10 @@
         <v>93</v>
       </c>
       <c r="U15" s="2" t="n">
-        <v>156.0</v>
+        <v>340.0</v>
       </c>
       <c r="V15" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="W15" s="2" t="b">
         <v>0</v>
@@ -5895,31 +5863,31 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E16" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="I16" s="2" t="s">
         <v>225</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>3.0</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>226</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>165</v>
@@ -5955,10 +5923,10 @@
         <v>93</v>
       </c>
       <c r="U16" s="2" t="n">
-        <v>318.0</v>
+        <v>1.0</v>
       </c>
       <c r="V16" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="W16" s="2" t="b">
         <v>0</v>
@@ -5990,28 +5958,28 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>227</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>228</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>174</v>
+        <v>228</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>93</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>163</v>
+        <v>193</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>229</v>
@@ -6050,10 +6018,10 @@
         <v>93</v>
       </c>
       <c r="U17" s="2" t="n">
-        <v>56.0</v>
+        <v>824.0</v>
       </c>
       <c r="V17" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="W17" s="2" t="b">
         <v>0</v>
@@ -6094,22 +6062,22 @@
         <v>95</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="E18" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>232</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>2.0</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>233</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>165</v>
@@ -6145,10 +6113,10 @@
         <v>93</v>
       </c>
       <c r="U18" s="2" t="n">
-        <v>596.0</v>
+        <v>318.0</v>
       </c>
       <c r="V18" s="2" t="n">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="W18" s="2" t="b">
         <v>0</v>
@@ -6180,31 +6148,31 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>234</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>235</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>236</v>
+        <v>169</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>93</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>2.0</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>165</v>
@@ -6240,10 +6208,10 @@
         <v>93</v>
       </c>
       <c r="U19" s="2" t="n">
-        <v>701.0</v>
+        <v>138.0</v>
       </c>
       <c r="V19" s="2" t="n">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="W19" s="2" t="b">
         <v>0</v>
@@ -6288,7 +6256,7 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="9.4453125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="14.7265625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="6.83984375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="16.22265625" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="13.59375" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="15.30078125" customWidth="true" bestFit="true"/>
@@ -6296,10 +6264,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2"/>
@@ -6308,16 +6276,16 @@
         <v>140</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>241</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="4">
@@ -6357,7 +6325,7 @@
     <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>18.0</v>
@@ -6456,7 +6424,7 @@
         <v>93</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>93</v>
@@ -6622,7 +6590,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>105</v>
@@ -6719,8 +6687,8 @@
       <c r="B6" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>247</v>
+      <c r="C6" s="10" t="s">
+        <v>93</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>93</v>
@@ -6811,8 +6779,8 @@
       <c r="B10" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>93</v>
+      <c r="C10" s="6" t="s">
+        <v>245</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>93</v>
@@ -6971,7 +6939,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>105</v>
@@ -6994,13 +6962,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>205</v>
+        <v>169</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>93</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>93</v>

</xml_diff>

<commit_message>
Add room tag sets
</commit_message>
<xml_diff>
--- a/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
+++ b/optaplanner-examples/data/conferencescheduling/unsolved/18talks-6timeslots-5rooms.xlsx
@@ -304,7 +304,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1493" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1493" uniqueCount="283">
   <si>
     <t>Conference name</t>
   </si>
@@ -879,9 +879,6 @@
     <t>jBPM</t>
   </si>
   <si>
-    <t>Large</t>
-  </si>
-  <si>
     <t>S06</t>
   </si>
   <si>
@@ -1012,9 +1009,6 @@
   </si>
   <si>
     <t>Tensorflow</t>
-  </si>
-  <si>
-    <t>Large, Recorded</t>
   </si>
   <si>
     <t>S17</t>
@@ -1902,7 +1896,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>106</v>
@@ -1974,7 +1968,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>106</v>
@@ -2000,10 +1994,10 @@
         <v>164</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>93</v>
@@ -2093,13 +2087,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>93</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>93</v>
@@ -2116,10 +2110,10 @@
     </row>
     <row r="4" ht="15.0" customHeight="true">
       <c r="A4" s="1" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>93</v>
@@ -2189,7 +2183,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>106</v>
@@ -2212,13 +2206,13 @@
     </row>
     <row r="3" ht="15.0" customHeight="true">
       <c r="A3" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>93</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>93</v>
@@ -2235,10 +2229,10 @@
     </row>
     <row r="4" ht="15.0" customHeight="true">
       <c r="A4" s="1" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>93</v>
@@ -2258,10 +2252,10 @@
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="1" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>93</v>
@@ -2357,10 +2351,10 @@
         <v>166</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>93</v>
@@ -2404,39 +2398,39 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="D3" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>264</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -2449,13 +2443,13 @@
         <v>7</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6">
@@ -2463,13 +2457,13 @@
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="7">
@@ -2477,13 +2471,13 @@
         <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="8">
@@ -2491,13 +2485,13 @@
         <v>16</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="9">
@@ -2505,13 +2499,13 @@
         <v>19</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="10">
@@ -2519,13 +2513,13 @@
         <v>24</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="11">
@@ -2533,13 +2527,13 @@
         <v>37</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="12">
@@ -2547,13 +2541,13 @@
         <v>31</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="13">
@@ -2561,13 +2555,13 @@
         <v>35</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="14">
@@ -2575,13 +2569,13 @@
         <v>29</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C14" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="15">
@@ -2589,13 +2583,13 @@
         <v>21</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="16">
@@ -2603,13 +2597,13 @@
         <v>40</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="17">
@@ -2617,13 +2611,13 @@
         <v>34</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="18">
@@ -2631,13 +2625,13 @@
         <v>39</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C18" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="19">
@@ -2645,13 +2639,13 @@
         <v>33</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C19" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="20">
@@ -2659,13 +2653,13 @@
         <v>41</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C20" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="21">
@@ -2673,13 +2667,13 @@
         <v>62</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C21" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="22">
@@ -2687,13 +2681,13 @@
         <v>78</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C22" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="23">
@@ -2701,13 +2695,13 @@
         <v>71</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C23" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="24">
@@ -2715,13 +2709,13 @@
         <v>80</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C24" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="25">
@@ -2729,13 +2723,13 @@
         <v>74</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C25" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="26">
@@ -2743,13 +2737,13 @@
         <v>82</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C26" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="27">
@@ -2757,13 +2751,13 @@
         <v>76</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C27" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="28">
@@ -2771,13 +2765,13 @@
         <v>83</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C28" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="29">
@@ -2785,13 +2779,13 @@
         <v>77</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C29" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="30">
@@ -2799,13 +2793,13 @@
         <v>60</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C30" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="31">
@@ -2813,13 +2807,13 @@
         <v>65</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C31" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="32">
@@ -2827,13 +2821,13 @@
         <v>69</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C32" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="33">
@@ -2841,13 +2835,13 @@
         <v>44</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C33" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="34">
@@ -2855,13 +2849,13 @@
         <v>67</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C34" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="35">
@@ -2869,13 +2863,13 @@
         <v>51</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C35" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="36">
@@ -2883,13 +2877,13 @@
         <v>47</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C36" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="37">
@@ -2897,13 +2891,13 @@
         <v>49</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C37" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="38">
@@ -2911,13 +2905,13 @@
         <v>58</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C38" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="39">
@@ -2925,13 +2919,13 @@
         <v>53</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C39" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="40">
@@ -2939,13 +2933,13 @@
         <v>56</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C40" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="41">
@@ -2953,13 +2947,13 @@
         <v>26</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C41" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="42"/>
@@ -2969,13 +2963,13 @@
         <v>49</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C44" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="45">
@@ -2985,10 +2979,10 @@
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
       <c r="F45" s="3" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="46">
@@ -2996,13 +2990,13 @@
         <v>47</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C46" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="47">
@@ -3012,10 +3006,10 @@
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
       <c r="F47" s="3" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="48">
@@ -3023,13 +3017,13 @@
         <v>56</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C48" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="49">
@@ -3039,10 +3033,10 @@
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
       <c r="F49" s="3" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="50">
@@ -3050,13 +3044,13 @@
         <v>58</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C50" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="51">
@@ -3064,13 +3058,13 @@
         <v>53</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C51" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="52">
@@ -3078,13 +3072,13 @@
         <v>24</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C52" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="53">
@@ -3092,13 +3086,13 @@
         <v>60</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C53" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="54">
@@ -3106,13 +3100,13 @@
         <v>62</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C54" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="55">
@@ -3120,13 +3114,13 @@
         <v>26</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C55" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="56">
@@ -3134,13 +3128,13 @@
         <v>65</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C56" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="57">
@@ -3148,13 +3142,13 @@
         <v>69</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C57" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="58">
@@ -3162,13 +3156,13 @@
         <v>44</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C58" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="59">
@@ -3176,13 +3170,13 @@
         <v>41</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C59" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="60">
@@ -3190,13 +3184,13 @@
         <v>10</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C60" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="61">
@@ -3204,13 +3198,13 @@
         <v>7</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C61" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="62">
@@ -3218,13 +3212,13 @@
         <v>67</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C62" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="63">
@@ -3232,13 +3226,13 @@
         <v>51</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C63" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="64">
@@ -3246,13 +3240,13 @@
         <v>16</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C64" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="65">
@@ -3260,13 +3254,13 @@
         <v>78</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C65" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="66">
@@ -3274,13 +3268,13 @@
         <v>71</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C66" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="67">
@@ -3288,13 +3282,13 @@
         <v>37</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C67" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="68">
@@ -3302,13 +3296,13 @@
         <v>31</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C68" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="69">
@@ -3316,13 +3310,13 @@
         <v>35</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C69" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="70">
@@ -3330,13 +3324,13 @@
         <v>29</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C70" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="71">
@@ -3344,13 +3338,13 @@
         <v>13</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C71" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="72">
@@ -3358,13 +3352,13 @@
         <v>80</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C72" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="73">
@@ -3372,13 +3366,13 @@
         <v>74</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C73" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="74">
@@ -3386,13 +3380,13 @@
         <v>21</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C74" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="75">
@@ -3400,13 +3394,13 @@
         <v>82</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C75" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="76">
@@ -3414,13 +3408,13 @@
         <v>76</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C76" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="77">
@@ -3428,13 +3422,13 @@
         <v>19</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C77" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="78">
@@ -3442,13 +3436,13 @@
         <v>40</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C78" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="79">
@@ -3456,13 +3450,13 @@
         <v>34</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C79" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="80">
@@ -3470,13 +3464,13 @@
         <v>39</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C80" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="81">
@@ -3484,13 +3478,13 @@
         <v>33</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C81" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="82">
@@ -3498,13 +3492,13 @@
         <v>83</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C82" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="83">
@@ -3512,13 +3506,13 @@
         <v>77</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C83" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -3559,7 +3553,7 @@
         <v>93</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" ht="45.0" customHeight="true">
@@ -3567,7 +3561,7 @@
         <v>107</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C3" s="2"/>
     </row>
@@ -4974,13 +4968,13 @@
         <v>93</v>
       </c>
       <c r="P3" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="R3" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="S3" s="2" t="s">
         <v>93</v>
@@ -5069,7 +5063,7 @@
         <v>93</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>93</v>
@@ -5164,7 +5158,7 @@
         <v>93</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>93</v>
@@ -5354,7 +5348,7 @@
         <v>93</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>191</v>
+        <v>93</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>93</v>
@@ -5404,10 +5398,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>193</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>95</v>
@@ -5428,7 +5422,7 @@
         <v>3.0</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>166</v>
@@ -5449,7 +5443,7 @@
         <v>93</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>191</v>
+        <v>93</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>93</v>
@@ -5499,10 +5493,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>196</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>95</v>
@@ -5511,10 +5505,10 @@
         <v>137</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>197</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>198</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>170</v>
@@ -5523,7 +5517,7 @@
         <v>3.0</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>166</v>
@@ -5544,7 +5538,7 @@
         <v>93</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>93</v>
@@ -5594,19 +5588,19 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>202</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>203</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>93</v>
@@ -5618,7 +5612,7 @@
         <v>3.0</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>166</v>
@@ -5639,7 +5633,7 @@
         <v>93</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>191</v>
+        <v>93</v>
       </c>
       <c r="Q10" s="2" t="s">
         <v>93</v>
@@ -5689,19 +5683,19 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>206</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>174</v>
@@ -5713,7 +5707,7 @@
         <v>3.0</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>166</v>
@@ -5784,16 +5778,16 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>209</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>210</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>163</v>
@@ -5808,7 +5802,7 @@
         <v>1.0</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>166</v>
@@ -5879,19 +5873,19 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>213</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>214</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>93</v>
@@ -5903,7 +5897,7 @@
         <v>3.0</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>166</v>
@@ -5924,7 +5918,7 @@
         <v>93</v>
       </c>
       <c r="P13" s="2" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>93</v>
@@ -5933,7 +5927,7 @@
         <v>93</v>
       </c>
       <c r="S13" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="T13" s="2" t="s">
         <v>93</v>
@@ -5974,10 +5968,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>218</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>219</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>95</v>
@@ -5986,7 +5980,7 @@
         <v>134</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>93</v>
@@ -5998,7 +5992,7 @@
         <v>3.0</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>166</v>
@@ -6069,10 +6063,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>223</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>95</v>
@@ -6093,7 +6087,7 @@
         <v>3.0</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>166</v>
@@ -6164,10 +6158,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>225</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>226</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>95</v>
@@ -6176,7 +6170,7 @@
         <v>136</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>93</v>
@@ -6188,7 +6182,7 @@
         <v>2.0</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>166</v>
@@ -6206,16 +6200,16 @@
         <v>93</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>93</v>
+        <v>113</v>
       </c>
       <c r="P16" s="2" t="s">
-        <v>191</v>
+        <v>93</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>93</v>
       </c>
       <c r="R16" s="2" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="S16" s="2" t="s">
         <v>93</v>
@@ -6259,16 +6253,16 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>229</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>230</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>179</v>
@@ -6283,7 +6277,7 @@
         <v>1.0</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>166</v>
@@ -6304,7 +6298,7 @@
         <v>93</v>
       </c>
       <c r="P17" s="2" t="s">
-        <v>191</v>
+        <v>93</v>
       </c>
       <c r="Q17" s="2" t="s">
         <v>93</v>
@@ -6354,10 +6348,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>233</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>234</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>95</v>
@@ -6378,7 +6372,7 @@
         <v>2.0</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>166</v>
@@ -6399,7 +6393,7 @@
         <v>93</v>
       </c>
       <c r="P18" s="2" t="s">
-        <v>236</v>
+        <v>93</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>93</v>
@@ -6449,19 +6443,19 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>93</v>
@@ -6473,7 +6467,7 @@
         <v>2.0</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>166</v>
@@ -6494,7 +6488,7 @@
         <v>93</v>
       </c>
       <c r="P19" s="2" t="s">
-        <v>236</v>
+        <v>93</v>
       </c>
       <c r="Q19" s="2" t="s">
         <v>93</v>
@@ -6565,10 +6559,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2"/>
@@ -6577,16 +6571,16 @@
         <v>141</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>243</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="4">
@@ -6626,7 +6620,7 @@
     <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>18.0</v>
@@ -6725,7 +6719,7 @@
         <v>93</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>93</v>
@@ -6814,7 +6808,7 @@
         <v>118</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -6888,7 +6882,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>106</v>
@@ -6914,7 +6908,7 @@
         <v>127</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -6933,7 +6927,7 @@
         <v>128</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -6978,7 +6972,7 @@
         <v>93</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>93</v>
@@ -7001,7 +6995,7 @@
         <v>93</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>93</v>
@@ -7231,7 +7225,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>106</v>
@@ -7257,10 +7251,10 @@
         <v>163</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>93</v>

</xml_diff>